<commit_message>
Revert "Add the Gateway and Diagnosis Validation"
This reverts commit 241e2089a41889967f6fe0ad016d500990d9fe31, reversing
changes made to 9b7dfdee383ce4011ee0284b552d2243b7c77f07.
</commit_message>
<xml_diff>
--- a/src/data/real_use_cases.xlsx
+++ b/src/data/real_use_cases.xlsx
@@ -9,7 +9,7 @@
     </mc:Choice>
   </mc:AlternateContent>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="28800" windowHeight="12300"/>
+    <workbookView xWindow="0" yWindow="0" windowWidth="28800" windowHeight="12300" activeTab="1"/>
   </bookViews>
   <sheets>
     <sheet name="Scripts" sheetId="1" r:id="rId1"/>
@@ -27,7 +27,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="259" uniqueCount="158">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="255" uniqueCount="156">
   <si>
     <t>Departement</t>
   </si>
@@ -118,9 +118,6 @@
     <t>Final Diagnosis</t>
   </si>
   <si>
-    <t>Unstable angina / acute coronary syndrome under evaluation.</t>
-  </si>
-  <si>
     <t>Plan of Care</t>
   </si>
   <si>
@@ -145,33 +142,18 @@
     <t>Expected</t>
   </si>
   <si>
-    <t>A – Airway</t>
-  </si>
-  <si>
     <t>Patent</t>
   </si>
   <si>
-    <t>B – Breathing</t>
-  </si>
-  <si>
     <t>Spontaneous breathing</t>
   </si>
   <si>
-    <t>C – Circulation</t>
-  </si>
-  <si>
     <t>Hemodynamically stabl</t>
   </si>
   <si>
-    <t>D – Disability</t>
-  </si>
-  <si>
     <t>No neurological abnormality reported</t>
   </si>
   <si>
-    <t>E – Exposure</t>
-  </si>
-  <si>
     <t>No significant abnormality reported.</t>
   </si>
   <si>
@@ -212,9 +194,6 @@
   </si>
   <si>
     <t>Patient is drowsy, pale, delirious, and has a disturbed conscious level. Laboratory findings showed anemia with hemoglobin 8.5 g/dL, elevated TLC, metabolic acidosis, and elevated renal function tests.</t>
-  </si>
-  <si>
-    <t>Acute confusional state with metabolic acidosis and renal impairment; possible acute kidney injury on top of chronic kidney disease, with sepsis/septic shock to be excluded.</t>
   </si>
   <si>
     <t>ICU admission. Close monitoring of conscious level, hemodynamic status, renal function, and acid-base status. Further infectious and metabolic workup. ICU consultant review. Infectious disease consultation for further evaluation and management.</t>
@@ -538,22 +517,6 @@
   </si>
   <si>
     <t>3 Months</t>
-  </si>
-  <si>
-    <r>
-      <t>Social / Marital / Family History</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="12"/>
-        <rFont val="Arial"/>
-        <family val="2"/>
-      </rPr>
-      <t> </t>
-    </r>
-  </si>
-  <si>
-    <t>Plan of Care (short/long term)</t>
   </si>
   <si>
     <t>Procedures Planned</t>
@@ -588,6 +551,37 @@
 No internal referrals were required.  
 The patient will return after three months for healing assessment and prosthetic restoration planning.  
 Retention priority is high.</t>
+  </si>
+  <si>
+    <t>Airway</t>
+  </si>
+  <si>
+    <t>Breathing</t>
+  </si>
+  <si>
+    <t>Circulation</t>
+  </si>
+  <si>
+    <t>Disability</t>
+  </si>
+  <si>
+    <t>Exposure</t>
+  </si>
+  <si>
+    <t>Differential Diagnoses</t>
+  </si>
+  <si>
+    <r>
+      <t>Social Family History</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t> </t>
+    </r>
   </si>
 </sst>
 </file>
@@ -800,7 +794,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="21">
+  <cellXfs count="20">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
@@ -821,12 +815,6 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="5" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="5" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="5" fillId="4" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
@@ -839,12 +827,6 @@
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
     <xf numFmtId="0" fontId="7" fillId="6" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
@@ -854,8 +836,17 @@
     <xf numFmtId="0" fontId="1" fillId="7" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="7" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
+    <xf numFmtId="0" fontId="3" fillId="5" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="5" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -1232,7 +1223,7 @@
         <v>4</v>
       </c>
       <c r="C9" s="5" t="s">
-        <v>157</v>
+        <v>148</v>
       </c>
     </row>
     <row r="10" spans="1:3" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
@@ -1291,52 +1282,52 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:B41"/>
+  <dimension ref="A1:B39"/>
   <sheetFormatPr defaultColWidth="22.140625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="2" max="2" width="79.28515625" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:2" ht="21" x14ac:dyDescent="0.25">
-      <c r="A1" s="8" t="s">
-        <v>46</v>
-      </c>
-      <c r="B1" s="9"/>
+      <c r="A1" s="15" t="s">
+        <v>40</v>
+      </c>
+      <c r="B1" s="16"/>
     </row>
     <row r="2" spans="1:2" ht="18.75" x14ac:dyDescent="0.25">
-      <c r="A2" s="10" t="s">
+      <c r="A2" s="8" t="s">
+        <v>32</v>
+      </c>
+      <c r="B2" s="8" t="s">
         <v>33</v>
       </c>
-      <c r="B2" s="10" t="s">
-        <v>34</v>
-      </c>
     </row>
     <row r="3" spans="1:2" ht="45" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A3" s="12" t="s">
+      <c r="A3" s="10" t="s">
         <v>12</v>
       </c>
-      <c r="B3" s="11" t="s">
+      <c r="B3" s="9" t="s">
         <v>13</v>
       </c>
     </row>
     <row r="4" spans="1:2" ht="45" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A4" s="13" t="s">
-        <v>45</v>
+      <c r="A4" s="11" t="s">
+        <v>154</v>
       </c>
       <c r="B4" s="6" t="s">
         <v>14</v>
       </c>
     </row>
     <row r="5" spans="1:2" ht="45" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A5" s="12" t="s">
+      <c r="A5" s="10" t="s">
         <v>15</v>
       </c>
-      <c r="B5" s="11" t="s">
+      <c r="B5" s="9" t="s">
         <v>16</v>
       </c>
     </row>
     <row r="6" spans="1:2" ht="45" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A6" s="13" t="s">
+      <c r="A6" s="11" t="s">
         <v>17</v>
       </c>
       <c r="B6" s="7" t="s">
@@ -1344,15 +1335,15 @@
       </c>
     </row>
     <row r="7" spans="1:2" ht="45" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A7" s="12" t="s">
+      <c r="A7" s="10" t="s">
         <v>18</v>
       </c>
-      <c r="B7" s="11" t="s">
+      <c r="B7" s="9" t="s">
         <v>16</v>
       </c>
     </row>
     <row r="8" spans="1:2" ht="45" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A8" s="13" t="s">
+      <c r="A8" s="11" t="s">
         <v>19</v>
       </c>
       <c r="B8" s="7" t="s">
@@ -1360,268 +1351,252 @@
       </c>
     </row>
     <row r="9" spans="1:2" ht="45" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A9" s="12" t="s">
+      <c r="A9" s="10" t="s">
         <v>21</v>
       </c>
-      <c r="B9" s="11" t="s">
+      <c r="B9" s="9" t="s">
         <v>22</v>
       </c>
     </row>
     <row r="10" spans="1:2" ht="45" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A10" s="16" t="s">
+      <c r="A10" s="12" t="s">
+        <v>149</v>
+      </c>
+      <c r="B10" s="13" t="s">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="11" spans="1:2" ht="45" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A11" s="10" t="s">
+        <v>150</v>
+      </c>
+      <c r="B11" s="9" t="s">
         <v>35</v>
       </c>
-      <c r="B10" s="17" t="s">
+    </row>
+    <row r="12" spans="1:2" ht="45" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A12" s="12" t="s">
+        <v>151</v>
+      </c>
+      <c r="B12" s="13" t="s">
         <v>36</v>
       </c>
     </row>
-    <row r="11" spans="1:2" ht="45" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A11" s="12" t="s">
+    <row r="13" spans="1:2" ht="45" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A13" s="10" t="s">
+        <v>152</v>
+      </c>
+      <c r="B13" s="9" t="s">
         <v>37</v>
       </c>
-      <c r="B11" s="11" t="s">
+    </row>
+    <row r="14" spans="1:2" ht="45" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A14" s="12" t="s">
+        <v>153</v>
+      </c>
+      <c r="B14" s="13" t="s">
         <v>38</v>
       </c>
     </row>
-    <row r="12" spans="1:2" ht="45" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A12" s="16" t="s">
-        <v>39</v>
-      </c>
-      <c r="B12" s="17" t="s">
-        <v>40</v>
-      </c>
-    </row>
-    <row r="13" spans="1:2" ht="45" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A13" s="12" t="s">
+    <row r="15" spans="1:2" ht="45" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A15" s="10" t="s">
+        <v>23</v>
+      </c>
+      <c r="B15" s="9" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="16" spans="1:2" ht="45" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A16" s="12" t="s">
+        <v>26</v>
+      </c>
+      <c r="B16" s="12" t="s">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="17" spans="1:2" ht="45" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A17" s="10" t="s">
+        <v>28</v>
+      </c>
+      <c r="B17" s="10" t="s">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="18" spans="1:2" ht="45" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A18" s="14" t="s">
+        <v>30</v>
+      </c>
+      <c r="B18" s="14" t="s">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="19" spans="1:2" ht="45" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A19" s="10" t="s">
+        <v>42</v>
+      </c>
+      <c r="B19" s="10" t="s">
+        <v>43</v>
+      </c>
+    </row>
+    <row r="20" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A20" s="17"/>
+      <c r="B20" s="17"/>
+    </row>
+    <row r="21" spans="1:2" ht="21" x14ac:dyDescent="0.25">
+      <c r="A21" s="15" t="s">
         <v>41</v>
       </c>
-      <c r="B13" s="11" t="s">
-        <v>42</v>
-      </c>
-    </row>
-    <row r="14" spans="1:2" ht="45" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A14" s="16" t="s">
-        <v>43</v>
-      </c>
-      <c r="B14" s="17" t="s">
+      <c r="B21" s="16"/>
+    </row>
+    <row r="22" spans="1:2" ht="18.75" x14ac:dyDescent="0.25">
+      <c r="A22" s="8" t="s">
+        <v>32</v>
+      </c>
+      <c r="B22" s="8" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="23" spans="1:2" ht="48" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A23" s="11" t="s">
+        <v>12</v>
+      </c>
+      <c r="B23" s="1" t="s">
         <v>44</v>
       </c>
     </row>
-    <row r="15" spans="1:2" ht="45" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A15" s="12" t="s">
-        <v>23</v>
-      </c>
-      <c r="B15" s="11" t="s">
-        <v>24</v>
-      </c>
-    </row>
-    <row r="16" spans="1:2" ht="45" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A16" s="16" t="s">
-        <v>25</v>
-      </c>
-      <c r="B16" s="17" t="s">
-        <v>26</v>
-      </c>
-    </row>
-    <row r="17" spans="1:2" ht="45" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A17" s="12" t="s">
-        <v>27</v>
-      </c>
-      <c r="B17" s="11" t="s">
-        <v>28</v>
-      </c>
-    </row>
-    <row r="18" spans="1:2" ht="45" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A18" s="16" t="s">
-        <v>29</v>
-      </c>
-      <c r="B18" s="17" t="s">
-        <v>30</v>
-      </c>
-    </row>
-    <row r="19" spans="1:2" ht="45" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A19" s="12" t="s">
-        <v>31</v>
-      </c>
-      <c r="B19" s="11" t="s">
-        <v>32</v>
-      </c>
-    </row>
-    <row r="20" spans="1:2" ht="45" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A20" s="18" t="s">
+    <row r="24" spans="1:2" ht="48" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A24" s="10" t="s">
+        <v>154</v>
+      </c>
+      <c r="B24" s="9" t="s">
+        <v>45</v>
+      </c>
+    </row>
+    <row r="25" spans="1:2" ht="48" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A25" s="11" t="s">
+        <v>15</v>
+      </c>
+      <c r="B25" s="1" t="s">
+        <v>46</v>
+      </c>
+    </row>
+    <row r="26" spans="1:2" ht="48" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A26" s="10" t="s">
+        <v>17</v>
+      </c>
+      <c r="B26" s="9" t="s">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="27" spans="1:2" ht="48" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A27" s="11" t="s">
+        <v>18</v>
+      </c>
+      <c r="B27" s="1" t="s">
         <v>48</v>
       </c>
-      <c r="B20" s="19" t="s">
+    </row>
+    <row r="28" spans="1:2" ht="48" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A28" s="10" t="s">
+        <v>19</v>
+      </c>
+      <c r="B28" s="9" t="s">
         <v>49</v>
       </c>
     </row>
-    <row r="21" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A21" s="14"/>
-      <c r="B21" s="14"/>
-    </row>
-    <row r="22" spans="1:2" ht="21" x14ac:dyDescent="0.25">
-      <c r="A22" s="8" t="s">
-        <v>47</v>
-      </c>
-      <c r="B22" s="9"/>
-    </row>
-    <row r="23" spans="1:2" ht="18.75" x14ac:dyDescent="0.25">
-      <c r="A23" s="10" t="s">
-        <v>33</v>
-      </c>
-      <c r="B23" s="10" t="s">
+    <row r="29" spans="1:2" ht="48" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A29" s="11" t="s">
+        <v>21</v>
+      </c>
+      <c r="B29" s="1" t="s">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="30" spans="1:2" ht="48" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A30" s="10" t="s">
+        <v>149</v>
+      </c>
+      <c r="B30" s="9" t="s">
         <v>34</v>
-      </c>
-    </row>
-    <row r="24" spans="1:2" ht="48" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A24" s="13" t="s">
-        <v>12</v>
-      </c>
-      <c r="B24" s="1" t="s">
-        <v>50</v>
-      </c>
-    </row>
-    <row r="25" spans="1:2" ht="48" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A25" s="12" t="s">
-        <v>45</v>
-      </c>
-      <c r="B25" s="11" t="s">
-        <v>51</v>
-      </c>
-    </row>
-    <row r="26" spans="1:2" ht="48" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A26" s="13" t="s">
-        <v>15</v>
-      </c>
-      <c r="B26" s="1" t="s">
-        <v>52</v>
-      </c>
-    </row>
-    <row r="27" spans="1:2" ht="48" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A27" s="12" t="s">
-        <v>17</v>
-      </c>
-      <c r="B27" s="11" t="s">
-        <v>53</v>
-      </c>
-    </row>
-    <row r="28" spans="1:2" ht="48" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A28" s="13" t="s">
-        <v>18</v>
-      </c>
-      <c r="B28" s="1" t="s">
-        <v>54</v>
-      </c>
-    </row>
-    <row r="29" spans="1:2" ht="48" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A29" s="12" t="s">
-        <v>19</v>
-      </c>
-      <c r="B29" s="11" t="s">
-        <v>55</v>
-      </c>
-    </row>
-    <row r="30" spans="1:2" ht="48" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A30" s="13" t="s">
-        <v>21</v>
-      </c>
-      <c r="B30" s="1" t="s">
-        <v>56</v>
       </c>
     </row>
     <row r="31" spans="1:2" ht="48" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A31" s="12" t="s">
-        <v>35</v>
-      </c>
-      <c r="B31" s="11" t="s">
-        <v>36</v>
+        <v>150</v>
+      </c>
+      <c r="B31" s="13" t="s">
+        <v>55</v>
       </c>
     </row>
     <row r="32" spans="1:2" ht="48" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A32" s="16" t="s">
-        <v>37</v>
-      </c>
-      <c r="B32" s="17" t="s">
-        <v>62</v>
+      <c r="A32" s="10" t="s">
+        <v>151</v>
+      </c>
+      <c r="B32" s="9" t="s">
+        <v>56</v>
       </c>
     </row>
     <row r="33" spans="1:2" ht="48" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A33" s="12" t="s">
-        <v>39</v>
-      </c>
-      <c r="B33" s="11" t="s">
-        <v>63</v>
+        <v>152</v>
+      </c>
+      <c r="B33" s="13" t="s">
+        <v>57</v>
       </c>
     </row>
     <row r="34" spans="1:2" ht="48" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A34" s="16" t="s">
-        <v>41</v>
-      </c>
-      <c r="B34" s="17" t="s">
-        <v>64</v>
+      <c r="A34" s="10" t="s">
+        <v>153</v>
+      </c>
+      <c r="B34" s="9" t="s">
+        <v>58</v>
       </c>
     </row>
     <row r="35" spans="1:2" ht="48" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A35" s="12" t="s">
-        <v>43</v>
-      </c>
-      <c r="B35" s="11" t="s">
-        <v>65</v>
+        <v>23</v>
+      </c>
+      <c r="B35" s="13" t="s">
+        <v>51</v>
       </c>
     </row>
     <row r="36" spans="1:2" ht="48" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A36" s="16" t="s">
-        <v>23</v>
-      </c>
-      <c r="B36" s="17" t="s">
-        <v>57</v>
+      <c r="A36" s="10" t="s">
+        <v>26</v>
+      </c>
+      <c r="B36" s="9" t="s">
+        <v>52</v>
       </c>
     </row>
     <row r="37" spans="1:2" ht="48" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A37" s="12" t="s">
-        <v>25</v>
-      </c>
-      <c r="B37" s="11" t="s">
-        <v>58</v>
+        <v>28</v>
+      </c>
+      <c r="B37" s="12" t="s">
+        <v>53</v>
       </c>
     </row>
     <row r="38" spans="1:2" ht="48" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A38" s="16" t="s">
-        <v>27</v>
-      </c>
-      <c r="B38" s="17" t="s">
-        <v>59</v>
+      <c r="A38" s="10" t="s">
+        <v>30</v>
+      </c>
+      <c r="B38" s="10" t="s">
+        <v>54</v>
       </c>
     </row>
     <row r="39" spans="1:2" ht="48" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A39" s="12" t="s">
-        <v>29</v>
-      </c>
-      <c r="B39" s="11" t="s">
-        <v>60</v>
-      </c>
-    </row>
-    <row r="40" spans="1:2" ht="48" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A40" s="16" t="s">
-        <v>31</v>
-      </c>
-      <c r="B40" s="17" t="s">
-        <v>61</v>
-      </c>
-    </row>
-    <row r="41" spans="1:2" ht="48" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A41" s="12" t="s">
-        <v>48</v>
-      </c>
-      <c r="B41" s="11" t="s">
-        <v>49</v>
+        <v>42</v>
+      </c>
+      <c r="B39" s="12" t="s">
+        <v>43</v>
       </c>
     </row>
   </sheetData>
   <mergeCells count="3">
     <mergeCell ref="A1:B1"/>
-    <mergeCell ref="A22:B22"/>
     <mergeCell ref="A21:B21"/>
+    <mergeCell ref="A20:B20"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" r:id="rId1"/>
@@ -1637,307 +1612,307 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:2" ht="21" x14ac:dyDescent="0.25">
-      <c r="A1" s="8" t="s">
+      <c r="A1" s="15" t="s">
+        <v>78</v>
+      </c>
+      <c r="B1" s="16"/>
+    </row>
+    <row r="2" spans="1:2" ht="18.75" x14ac:dyDescent="0.25">
+      <c r="A2" s="8" t="s">
+        <v>32</v>
+      </c>
+      <c r="B2" s="8" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="3" spans="1:2" ht="45" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A3" s="10" t="s">
+        <v>12</v>
+      </c>
+      <c r="B3" s="9" t="s">
+        <v>59</v>
+      </c>
+    </row>
+    <row r="4" spans="1:2" ht="45" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A4" s="11" t="s">
+        <v>15</v>
+      </c>
+      <c r="B4" s="7" t="s">
+        <v>93</v>
+      </c>
+    </row>
+    <row r="5" spans="1:2" ht="45" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A5" s="10" t="s">
+        <v>17</v>
+      </c>
+      <c r="B5" s="9" t="s">
+        <v>91</v>
+      </c>
+    </row>
+    <row r="6" spans="1:2" ht="45" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A6" s="11" t="s">
+        <v>18</v>
+      </c>
+      <c r="B6" s="7" t="s">
+        <v>92</v>
+      </c>
+    </row>
+    <row r="7" spans="1:2" ht="45" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A7" s="10" t="s">
+        <v>60</v>
+      </c>
+      <c r="B7" s="9" t="s">
+        <v>61</v>
+      </c>
+    </row>
+    <row r="8" spans="1:2" ht="45" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A8" s="11" t="s">
+        <v>90</v>
+      </c>
+      <c r="B8" s="7" t="s">
+        <v>62</v>
+      </c>
+    </row>
+    <row r="9" spans="1:2" ht="45" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A9" s="10" t="s">
+        <v>63</v>
+      </c>
+      <c r="B9" s="9" t="s">
+        <v>64</v>
+      </c>
+    </row>
+    <row r="10" spans="1:2" ht="45" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A10" s="11" t="s">
+        <v>65</v>
+      </c>
+      <c r="B10" s="7" t="s">
+        <v>66</v>
+      </c>
+    </row>
+    <row r="11" spans="1:2" ht="45" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A11" s="10" t="s">
+        <v>155</v>
+      </c>
+      <c r="B11" s="9" t="s">
+        <v>67</v>
+      </c>
+    </row>
+    <row r="12" spans="1:2" ht="45" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A12" s="11" t="s">
+        <v>146</v>
+      </c>
+      <c r="B12" s="7" t="s">
+        <v>68</v>
+      </c>
+    </row>
+    <row r="13" spans="1:2" ht="45" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A13" s="10" t="s">
+        <v>26</v>
+      </c>
+      <c r="B13" s="9" t="s">
+        <v>69</v>
+      </c>
+    </row>
+    <row r="14" spans="1:2" ht="45" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A14" s="11" t="s">
+        <v>143</v>
+      </c>
+      <c r="B14" s="7" t="s">
+        <v>70</v>
+      </c>
+    </row>
+    <row r="15" spans="1:2" ht="45" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A15" s="10" t="s">
+        <v>71</v>
+      </c>
+      <c r="B15" s="9" t="s">
+        <v>72</v>
+      </c>
+    </row>
+    <row r="16" spans="1:2" ht="45" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A16" s="11" t="s">
+        <v>144</v>
+      </c>
+      <c r="B16" s="7" t="s">
+        <v>73</v>
+      </c>
+    </row>
+    <row r="17" spans="1:2" ht="45" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A17" s="10" t="s">
+        <v>74</v>
+      </c>
+      <c r="B17" s="9" t="s">
+        <v>75</v>
+      </c>
+    </row>
+    <row r="18" spans="1:2" ht="45" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A18" s="11" t="s">
+        <v>147</v>
+      </c>
+      <c r="B18" s="7" t="s">
+        <v>76</v>
+      </c>
+    </row>
+    <row r="19" spans="1:2" ht="45" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A19" s="10" t="s">
+        <v>145</v>
+      </c>
+      <c r="B19" s="9" t="s">
+        <v>77</v>
+      </c>
+    </row>
+    <row r="20" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A20" s="18"/>
+      <c r="B20" s="18"/>
+    </row>
+    <row r="21" spans="1:2" ht="21" x14ac:dyDescent="0.25">
+      <c r="A21" s="15" t="s">
+        <v>79</v>
+      </c>
+      <c r="B21" s="16"/>
+    </row>
+    <row r="22" spans="1:2" ht="18.75" x14ac:dyDescent="0.25">
+      <c r="A22" s="8" t="s">
+        <v>32</v>
+      </c>
+      <c r="B22" s="8" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="23" spans="1:2" ht="45" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A23" s="10" t="s">
+        <v>12</v>
+      </c>
+      <c r="B23" s="9" t="s">
+        <v>80</v>
+      </c>
+    </row>
+    <row r="24" spans="1:2" ht="45" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A24" s="11" t="s">
+        <v>15</v>
+      </c>
+      <c r="B24" s="7" t="s">
+        <v>93</v>
+      </c>
+    </row>
+    <row r="25" spans="1:2" ht="45" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A25" s="10" t="s">
+        <v>17</v>
+      </c>
+      <c r="B25" s="9" t="s">
+        <v>91</v>
+      </c>
+    </row>
+    <row r="26" spans="1:2" ht="45" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A26" s="11" t="s">
+        <v>18</v>
+      </c>
+      <c r="B26" s="7" t="s">
+        <v>94</v>
+      </c>
+    </row>
+    <row r="27" spans="1:2" ht="45" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A27" s="10" t="s">
+        <v>60</v>
+      </c>
+      <c r="B27" s="9" t="s">
+        <v>61</v>
+      </c>
+    </row>
+    <row r="28" spans="1:2" ht="45" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A28" s="11" t="s">
+        <v>90</v>
+      </c>
+      <c r="B28" s="13" t="s">
+        <v>81</v>
+      </c>
+    </row>
+    <row r="29" spans="1:2" ht="45" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A29" s="10" t="s">
+        <v>63</v>
+      </c>
+      <c r="B29" s="9" t="s">
+        <v>82</v>
+      </c>
+    </row>
+    <row r="30" spans="1:2" ht="45" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A30" s="11" t="s">
+        <v>65</v>
+      </c>
+      <c r="B30" s="13" t="s">
+        <v>66</v>
+      </c>
+    </row>
+    <row r="31" spans="1:2" ht="45" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A31" s="10" t="s">
+        <v>155</v>
+      </c>
+      <c r="B31" s="9" t="s">
+        <v>83</v>
+      </c>
+    </row>
+    <row r="32" spans="1:2" ht="45" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A32" s="11" t="s">
+        <v>146</v>
+      </c>
+      <c r="B32" s="13" t="s">
+        <v>84</v>
+      </c>
+    </row>
+    <row r="33" spans="1:2" ht="45" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A33" s="10" t="s">
+        <v>26</v>
+      </c>
+      <c r="B33" s="9" t="s">
         <v>85</v>
       </c>
-      <c r="B1" s="9"/>
-    </row>
-    <row r="2" spans="1:2" ht="18.75" x14ac:dyDescent="0.25">
-      <c r="A2" s="10" t="s">
-        <v>33</v>
-      </c>
-      <c r="B2" s="10" t="s">
-        <v>34</v>
-      </c>
-    </row>
-    <row r="3" spans="1:2" ht="45" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A3" s="12" t="s">
-        <v>12</v>
-      </c>
-      <c r="B3" s="11" t="s">
-        <v>66</v>
-      </c>
-    </row>
-    <row r="4" spans="1:2" ht="45" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A4" s="13" t="s">
-        <v>15</v>
-      </c>
-      <c r="B4" s="7" t="s">
-        <v>100</v>
-      </c>
-    </row>
-    <row r="5" spans="1:2" ht="45" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A5" s="12" t="s">
-        <v>17</v>
-      </c>
-      <c r="B5" s="11" t="s">
-        <v>98</v>
-      </c>
-    </row>
-    <row r="6" spans="1:2" ht="45" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A6" s="13" t="s">
-        <v>18</v>
-      </c>
-      <c r="B6" s="7" t="s">
-        <v>99</v>
-      </c>
-    </row>
-    <row r="7" spans="1:2" ht="45" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A7" s="12" t="s">
-        <v>67</v>
-      </c>
-      <c r="B7" s="11" t="s">
-        <v>68</v>
-      </c>
-    </row>
-    <row r="8" spans="1:2" ht="45" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A8" s="13" t="s">
-        <v>97</v>
-      </c>
-      <c r="B8" s="7" t="s">
-        <v>69</v>
-      </c>
-    </row>
-    <row r="9" spans="1:2" ht="45" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A9" s="12" t="s">
-        <v>70</v>
-      </c>
-      <c r="B9" s="11" t="s">
+    </row>
+    <row r="34" spans="1:2" ht="45" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A34" s="11" t="s">
+        <v>143</v>
+      </c>
+      <c r="B34" s="13" t="s">
+        <v>86</v>
+      </c>
+    </row>
+    <row r="35" spans="1:2" ht="45" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A35" s="10" t="s">
         <v>71</v>
       </c>
-    </row>
-    <row r="10" spans="1:2" ht="45" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A10" s="13" t="s">
-        <v>72</v>
-      </c>
-      <c r="B10" s="7" t="s">
-        <v>73</v>
-      </c>
-    </row>
-    <row r="11" spans="1:2" ht="45" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A11" s="12" t="s">
-        <v>150</v>
-      </c>
-      <c r="B11" s="11" t="s">
+      <c r="B35" s="9" t="s">
+        <v>87</v>
+      </c>
+    </row>
+    <row r="36" spans="1:2" ht="45" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A36" s="11" t="s">
+        <v>144</v>
+      </c>
+      <c r="B36" s="13" t="s">
+        <v>88</v>
+      </c>
+    </row>
+    <row r="37" spans="1:2" ht="45" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A37" s="10" t="s">
         <v>74</v>
       </c>
-    </row>
-    <row r="12" spans="1:2" ht="45" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A12" s="13" t="s">
-        <v>155</v>
-      </c>
-      <c r="B12" s="7" t="s">
-        <v>75</v>
-      </c>
-    </row>
-    <row r="13" spans="1:2" ht="45" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A13" s="12" t="s">
-        <v>151</v>
-      </c>
-      <c r="B13" s="11" t="s">
+      <c r="B37" s="9" t="s">
+        <v>89</v>
+      </c>
+    </row>
+    <row r="38" spans="1:2" ht="45" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A38" s="11" t="s">
+        <v>147</v>
+      </c>
+      <c r="B38" s="13" t="s">
         <v>76</v>
       </c>
     </row>
-    <row r="14" spans="1:2" ht="45" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A14" s="13" t="s">
-        <v>152</v>
-      </c>
-      <c r="B14" s="7" t="s">
+    <row r="39" spans="1:2" ht="45" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A39" s="10" t="s">
+        <v>145</v>
+      </c>
+      <c r="B39" s="9" t="s">
         <v>77</v>
-      </c>
-    </row>
-    <row r="15" spans="1:2" ht="45" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A15" s="12" t="s">
-        <v>78</v>
-      </c>
-      <c r="B15" s="11" t="s">
-        <v>79</v>
-      </c>
-    </row>
-    <row r="16" spans="1:2" ht="45" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A16" s="13" t="s">
-        <v>153</v>
-      </c>
-      <c r="B16" s="7" t="s">
-        <v>80</v>
-      </c>
-    </row>
-    <row r="17" spans="1:2" ht="45" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A17" s="12" t="s">
-        <v>81</v>
-      </c>
-      <c r="B17" s="11" t="s">
-        <v>82</v>
-      </c>
-    </row>
-    <row r="18" spans="1:2" ht="45" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A18" s="13" t="s">
-        <v>156</v>
-      </c>
-      <c r="B18" s="7" t="s">
-        <v>83</v>
-      </c>
-    </row>
-    <row r="19" spans="1:2" ht="45" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A19" s="12" t="s">
-        <v>154</v>
-      </c>
-      <c r="B19" s="11" t="s">
-        <v>84</v>
-      </c>
-    </row>
-    <row r="20" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A20" s="15"/>
-      <c r="B20" s="15"/>
-    </row>
-    <row r="21" spans="1:2" ht="21" x14ac:dyDescent="0.25">
-      <c r="A21" s="8" t="s">
-        <v>86</v>
-      </c>
-      <c r="B21" s="9"/>
-    </row>
-    <row r="22" spans="1:2" ht="18.75" x14ac:dyDescent="0.25">
-      <c r="A22" s="10" t="s">
-        <v>33</v>
-      </c>
-      <c r="B22" s="10" t="s">
-        <v>34</v>
-      </c>
-    </row>
-    <row r="23" spans="1:2" ht="45" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A23" s="12" t="s">
-        <v>12</v>
-      </c>
-      <c r="B23" s="11" t="s">
-        <v>87</v>
-      </c>
-    </row>
-    <row r="24" spans="1:2" ht="45" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A24" s="13" t="s">
-        <v>15</v>
-      </c>
-      <c r="B24" s="7" t="s">
-        <v>100</v>
-      </c>
-    </row>
-    <row r="25" spans="1:2" ht="45" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A25" s="12" t="s">
-        <v>17</v>
-      </c>
-      <c r="B25" s="11" t="s">
-        <v>98</v>
-      </c>
-    </row>
-    <row r="26" spans="1:2" ht="45" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A26" s="13" t="s">
-        <v>18</v>
-      </c>
-      <c r="B26" s="7" t="s">
-        <v>101</v>
-      </c>
-    </row>
-    <row r="27" spans="1:2" ht="45" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A27" s="12" t="s">
-        <v>67</v>
-      </c>
-      <c r="B27" s="11" t="s">
-        <v>68</v>
-      </c>
-    </row>
-    <row r="28" spans="1:2" ht="45" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A28" s="13" t="s">
-        <v>97</v>
-      </c>
-      <c r="B28" s="17" t="s">
-        <v>88</v>
-      </c>
-    </row>
-    <row r="29" spans="1:2" ht="45" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A29" s="12" t="s">
-        <v>70</v>
-      </c>
-      <c r="B29" s="11" t="s">
-        <v>89</v>
-      </c>
-    </row>
-    <row r="30" spans="1:2" ht="45" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A30" s="13" t="s">
-        <v>72</v>
-      </c>
-      <c r="B30" s="17" t="s">
-        <v>73</v>
-      </c>
-    </row>
-    <row r="31" spans="1:2" ht="45" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A31" s="12" t="s">
-        <v>150</v>
-      </c>
-      <c r="B31" s="11" t="s">
-        <v>90</v>
-      </c>
-    </row>
-    <row r="32" spans="1:2" ht="45" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A32" s="13" t="s">
-        <v>155</v>
-      </c>
-      <c r="B32" s="17" t="s">
-        <v>91</v>
-      </c>
-    </row>
-    <row r="33" spans="1:2" ht="45" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A33" s="12" t="s">
-        <v>151</v>
-      </c>
-      <c r="B33" s="11" t="s">
-        <v>92</v>
-      </c>
-    </row>
-    <row r="34" spans="1:2" ht="45" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A34" s="13" t="s">
-        <v>152</v>
-      </c>
-      <c r="B34" s="17" t="s">
-        <v>93</v>
-      </c>
-    </row>
-    <row r="35" spans="1:2" ht="45" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A35" s="12" t="s">
-        <v>78</v>
-      </c>
-      <c r="B35" s="11" t="s">
-        <v>94</v>
-      </c>
-    </row>
-    <row r="36" spans="1:2" ht="45" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A36" s="13" t="s">
-        <v>153</v>
-      </c>
-      <c r="B36" s="17" t="s">
-        <v>95</v>
-      </c>
-    </row>
-    <row r="37" spans="1:2" ht="45" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A37" s="12" t="s">
-        <v>81</v>
-      </c>
-      <c r="B37" s="11" t="s">
-        <v>96</v>
-      </c>
-    </row>
-    <row r="38" spans="1:2" ht="45" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A38" s="13" t="s">
-        <v>156</v>
-      </c>
-      <c r="B38" s="17" t="s">
-        <v>83</v>
-      </c>
-    </row>
-    <row r="39" spans="1:2" ht="45" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A39" s="12" t="s">
-        <v>154</v>
-      </c>
-      <c r="B39" s="11" t="s">
-        <v>84</v>
       </c>
     </row>
   </sheetData>
@@ -1961,355 +1936,355 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:2" ht="21" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="8" t="s">
+      <c r="A1" s="15" t="s">
+        <v>95</v>
+      </c>
+      <c r="B1" s="16"/>
+    </row>
+    <row r="2" spans="1:2" ht="18.75" x14ac:dyDescent="0.25">
+      <c r="A2" s="8" t="s">
+        <v>32</v>
+      </c>
+      <c r="B2" s="8" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="3" spans="1:2" ht="45" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A3" s="10" t="s">
+        <v>96</v>
+      </c>
+      <c r="B3" s="9" t="s">
+        <v>97</v>
+      </c>
+    </row>
+    <row r="4" spans="1:2" ht="45" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A4" s="11" t="s">
+        <v>98</v>
+      </c>
+      <c r="B4" s="7" t="s">
+        <v>99</v>
+      </c>
+    </row>
+    <row r="5" spans="1:2" ht="45" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A5" s="10" t="s">
+        <v>12</v>
+      </c>
+      <c r="B5" s="9" t="s">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="6" spans="1:2" ht="45" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A6" s="11" t="s">
+        <v>39</v>
+      </c>
+      <c r="B6" s="7" t="s">
+        <v>101</v>
+      </c>
+    </row>
+    <row r="7" spans="1:2" ht="45" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A7" s="10" t="s">
+        <v>25</v>
+      </c>
+      <c r="B7" s="9" t="s">
         <v>102</v>
       </c>
-      <c r="B1" s="9"/>
-    </row>
-    <row r="2" spans="1:2" ht="18.75" x14ac:dyDescent="0.25">
-      <c r="A2" s="10" t="s">
+    </row>
+    <row r="8" spans="1:2" ht="45" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A8" s="11" t="s">
+        <v>103</v>
+      </c>
+      <c r="B8" s="7" t="s">
+        <v>104</v>
+      </c>
+    </row>
+    <row r="9" spans="1:2" ht="45" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A9" s="10" t="s">
+        <v>105</v>
+      </c>
+      <c r="B9" s="9" t="s">
+        <v>106</v>
+      </c>
+    </row>
+    <row r="10" spans="1:2" ht="45" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A10" s="11" t="s">
+        <v>107</v>
+      </c>
+      <c r="B10" s="7" t="s">
+        <v>108</v>
+      </c>
+    </row>
+    <row r="11" spans="1:2" ht="45" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A11" s="10" t="s">
+        <v>109</v>
+      </c>
+      <c r="B11" s="9" t="s">
+        <v>110</v>
+      </c>
+    </row>
+    <row r="12" spans="1:2" ht="45" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A12" s="11" t="s">
+        <v>111</v>
+      </c>
+      <c r="B12" s="7" t="s">
+        <v>112</v>
+      </c>
+    </row>
+    <row r="13" spans="1:2" ht="45" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A13" s="10" t="s">
+        <v>113</v>
+      </c>
+      <c r="B13" s="9" t="s">
+        <v>112</v>
+      </c>
+    </row>
+    <row r="14" spans="1:2" ht="45" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A14" s="11" t="s">
+        <v>114</v>
+      </c>
+      <c r="B14" s="7" t="s">
+        <v>115</v>
+      </c>
+    </row>
+    <row r="15" spans="1:2" ht="45" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A15" s="10" t="s">
+        <v>116</v>
+      </c>
+      <c r="B15" s="9" t="s">
+        <v>117</v>
+      </c>
+    </row>
+    <row r="16" spans="1:2" ht="45" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A16" s="11" t="s">
+        <v>118</v>
+      </c>
+      <c r="B16" s="7" t="s">
+        <v>119</v>
+      </c>
+    </row>
+    <row r="17" spans="1:2" ht="45" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A17" s="10" t="s">
+        <v>120</v>
+      </c>
+      <c r="B17" s="9" t="s">
+        <v>115</v>
+      </c>
+    </row>
+    <row r="18" spans="1:2" ht="45" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A18" s="12" t="s">
+        <v>121</v>
+      </c>
+      <c r="B18" s="13" t="s">
+        <v>122</v>
+      </c>
+    </row>
+    <row r="19" spans="1:2" ht="45" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A19" s="10" t="s">
+        <v>123</v>
+      </c>
+      <c r="B19" s="9" t="s">
+        <v>104</v>
+      </c>
+    </row>
+    <row r="20" spans="1:2" ht="45" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A20" s="12" t="s">
+        <v>124</v>
+      </c>
+      <c r="B20" s="13" t="s">
+        <v>125</v>
+      </c>
+    </row>
+    <row r="21" spans="1:2" ht="45" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A21" s="10" t="s">
+        <v>126</v>
+      </c>
+      <c r="B21" s="9" t="s">
+        <v>127</v>
+      </c>
+    </row>
+    <row r="22" spans="1:2" ht="45" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A22" s="12" t="s">
+        <v>128</v>
+      </c>
+      <c r="B22" s="13" t="s">
+        <v>129</v>
+      </c>
+    </row>
+    <row r="23" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A23" s="19"/>
+      <c r="B23" s="19"/>
+    </row>
+    <row r="24" spans="1:2" ht="21" x14ac:dyDescent="0.25">
+      <c r="A24" s="15" t="s">
+        <v>130</v>
+      </c>
+      <c r="B24" s="16"/>
+    </row>
+    <row r="25" spans="1:2" ht="18.75" x14ac:dyDescent="0.25">
+      <c r="A25" s="8" t="s">
+        <v>32</v>
+      </c>
+      <c r="B25" s="8" t="s">
         <v>33</v>
       </c>
-      <c r="B2" s="10" t="s">
-        <v>34</v>
-      </c>
-    </row>
-    <row r="3" spans="1:2" ht="45" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A3" s="12" t="s">
+    </row>
+    <row r="26" spans="1:2" ht="45" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A26" s="10" t="s">
+        <v>96</v>
+      </c>
+      <c r="B26" s="9" t="s">
+        <v>115</v>
+      </c>
+    </row>
+    <row r="27" spans="1:2" ht="45" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A27" s="11" t="s">
+        <v>98</v>
+      </c>
+      <c r="B27" s="7" t="s">
+        <v>131</v>
+      </c>
+    </row>
+    <row r="28" spans="1:2" ht="45" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A28" s="10" t="s">
+        <v>12</v>
+      </c>
+      <c r="B28" s="9" t="s">
+        <v>132</v>
+      </c>
+    </row>
+    <row r="29" spans="1:2" ht="45" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A29" s="11" t="s">
+        <v>39</v>
+      </c>
+      <c r="B29" s="7" t="s">
+        <v>133</v>
+      </c>
+    </row>
+    <row r="30" spans="1:2" ht="45" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A30" s="10" t="s">
+        <v>25</v>
+      </c>
+      <c r="B30" s="9" t="s">
+        <v>134</v>
+      </c>
+    </row>
+    <row r="31" spans="1:2" ht="45" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A31" s="11" t="s">
         <v>103</v>
       </c>
-      <c r="B3" s="11" t="s">
-        <v>104</v>
-      </c>
-    </row>
-    <row r="4" spans="1:2" ht="45" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A4" s="13" t="s">
+      <c r="B31" s="7" t="s">
+        <v>135</v>
+      </c>
+    </row>
+    <row r="32" spans="1:2" ht="45" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A32" s="10" t="s">
         <v>105</v>
       </c>
-      <c r="B4" s="7" t="s">
-        <v>106</v>
-      </c>
-    </row>
-    <row r="5" spans="1:2" ht="45" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A5" s="12" t="s">
-        <v>12</v>
-      </c>
-      <c r="B5" s="11" t="s">
+      <c r="B32" s="9" t="s">
+        <v>136</v>
+      </c>
+    </row>
+    <row r="33" spans="1:2" ht="45" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A33" s="11" t="s">
         <v>107</v>
       </c>
-    </row>
-    <row r="6" spans="1:2" ht="45" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A6" s="13" t="s">
-        <v>45</v>
-      </c>
-      <c r="B6" s="7" t="s">
-        <v>108</v>
-      </c>
-    </row>
-    <row r="7" spans="1:2" ht="45" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A7" s="12" t="s">
-        <v>25</v>
-      </c>
-      <c r="B7" s="11" t="s">
+      <c r="B33" s="7" t="s">
+        <v>137</v>
+      </c>
+    </row>
+    <row r="34" spans="1:2" ht="45" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A34" s="10" t="s">
         <v>109</v>
       </c>
-    </row>
-    <row r="8" spans="1:2" ht="45" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A8" s="13" t="s">
-        <v>110</v>
-      </c>
-      <c r="B8" s="7" t="s">
+      <c r="B34" s="9" t="s">
+        <v>138</v>
+      </c>
+    </row>
+    <row r="35" spans="1:2" ht="45" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A35" s="11" t="s">
         <v>111</v>
       </c>
-    </row>
-    <row r="9" spans="1:2" ht="45" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A9" s="12" t="s">
+      <c r="B35" s="7" t="s">
         <v>112</v>
       </c>
-      <c r="B9" s="11" t="s">
+    </row>
+    <row r="36" spans="1:2" ht="45" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A36" s="10" t="s">
         <v>113</v>
       </c>
-    </row>
-    <row r="10" spans="1:2" ht="45" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A10" s="13" t="s">
+      <c r="B36" s="9" t="s">
+        <v>112</v>
+      </c>
+    </row>
+    <row r="37" spans="1:2" ht="45" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A37" s="11" t="s">
         <v>114</v>
       </c>
-      <c r="B10" s="7" t="s">
+      <c r="B37" s="7" t="s">
         <v>115</v>
       </c>
     </row>
-    <row r="11" spans="1:2" ht="45" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A11" s="12" t="s">
+    <row r="38" spans="1:2" ht="45" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A38" s="10" t="s">
         <v>116</v>
       </c>
-      <c r="B11" s="11" t="s">
-        <v>117</v>
-      </c>
-    </row>
-    <row r="12" spans="1:2" ht="45" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A12" s="13" t="s">
+      <c r="B38" s="9" t="s">
+        <v>139</v>
+      </c>
+    </row>
+    <row r="39" spans="1:2" ht="45" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A39" s="11" t="s">
         <v>118</v>
       </c>
-      <c r="B12" s="7" t="s">
-        <v>119</v>
-      </c>
-    </row>
-    <row r="13" spans="1:2" ht="45" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A13" s="12" t="s">
+      <c r="B39" s="7" t="s">
+        <v>140</v>
+      </c>
+    </row>
+    <row r="40" spans="1:2" ht="45" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A40" s="10" t="s">
         <v>120</v>
       </c>
-      <c r="B13" s="11" t="s">
-        <v>119</v>
-      </c>
-    </row>
-    <row r="14" spans="1:2" ht="45" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A14" s="13" t="s">
+      <c r="B40" s="9" t="s">
+        <v>112</v>
+      </c>
+    </row>
+    <row r="41" spans="1:2" ht="45" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A41" s="11" t="s">
         <v>121</v>
       </c>
-      <c r="B14" s="7" t="s">
+      <c r="B41" s="7" t="s">
         <v>122</v>
       </c>
     </row>
-    <row r="15" spans="1:2" ht="45" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A15" s="12" t="s">
+    <row r="42" spans="1:2" ht="45" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A42" s="10" t="s">
         <v>123</v>
       </c>
-      <c r="B15" s="11" t="s">
+      <c r="B42" s="9" t="s">
+        <v>135</v>
+      </c>
+    </row>
+    <row r="43" spans="1:2" ht="45" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A43" s="11" t="s">
         <v>124</v>
       </c>
-    </row>
-    <row r="16" spans="1:2" ht="45" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A16" s="13" t="s">
-        <v>125</v>
-      </c>
-      <c r="B16" s="7" t="s">
+      <c r="B43" s="7" t="s">
+        <v>141</v>
+      </c>
+    </row>
+    <row r="44" spans="1:2" ht="45" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A44" s="10" t="s">
         <v>126</v>
       </c>
-    </row>
-    <row r="17" spans="1:2" ht="45" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A17" s="12" t="s">
+      <c r="B44" s="9" t="s">
         <v>127</v>
       </c>
-      <c r="B17" s="11" t="s">
-        <v>122</v>
-      </c>
-    </row>
-    <row r="18" spans="1:2" ht="45" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A18" s="16" t="s">
+    </row>
+    <row r="45" spans="1:2" ht="45" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A45" s="11" t="s">
         <v>128</v>
       </c>
-      <c r="B18" s="17" t="s">
-        <v>129</v>
-      </c>
-    </row>
-    <row r="19" spans="1:2" ht="45" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A19" s="12" t="s">
-        <v>130</v>
-      </c>
-      <c r="B19" s="11" t="s">
-        <v>111</v>
-      </c>
-    </row>
-    <row r="20" spans="1:2" ht="45" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A20" s="16" t="s">
-        <v>131</v>
-      </c>
-      <c r="B20" s="17" t="s">
-        <v>132</v>
-      </c>
-    </row>
-    <row r="21" spans="1:2" ht="45" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A21" s="12" t="s">
-        <v>133</v>
-      </c>
-      <c r="B21" s="11" t="s">
-        <v>134</v>
-      </c>
-    </row>
-    <row r="22" spans="1:2" ht="45" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A22" s="16" t="s">
-        <v>135</v>
-      </c>
-      <c r="B22" s="17" t="s">
-        <v>136</v>
-      </c>
-    </row>
-    <row r="23" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A23" s="20"/>
-      <c r="B23" s="20"/>
-    </row>
-    <row r="24" spans="1:2" ht="21" x14ac:dyDescent="0.25">
-      <c r="A24" s="8" t="s">
-        <v>137</v>
-      </c>
-      <c r="B24" s="9"/>
-    </row>
-    <row r="25" spans="1:2" ht="18.75" x14ac:dyDescent="0.25">
-      <c r="A25" s="10" t="s">
-        <v>33</v>
-      </c>
-      <c r="B25" s="10" t="s">
-        <v>34</v>
-      </c>
-    </row>
-    <row r="26" spans="1:2" ht="45" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A26" s="12" t="s">
-        <v>103</v>
-      </c>
-      <c r="B26" s="11" t="s">
-        <v>122</v>
-      </c>
-    </row>
-    <row r="27" spans="1:2" ht="45" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A27" s="13" t="s">
-        <v>105</v>
-      </c>
-      <c r="B27" s="7" t="s">
-        <v>138</v>
-      </c>
-    </row>
-    <row r="28" spans="1:2" ht="45" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A28" s="12" t="s">
-        <v>12</v>
-      </c>
-      <c r="B28" s="11" t="s">
-        <v>139</v>
-      </c>
-    </row>
-    <row r="29" spans="1:2" ht="45" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A29" s="13" t="s">
-        <v>45</v>
-      </c>
-      <c r="B29" s="7" t="s">
-        <v>140</v>
-      </c>
-    </row>
-    <row r="30" spans="1:2" ht="45" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A30" s="12" t="s">
-        <v>25</v>
-      </c>
-      <c r="B30" s="11" t="s">
-        <v>141</v>
-      </c>
-    </row>
-    <row r="31" spans="1:2" ht="45" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A31" s="13" t="s">
-        <v>110</v>
-      </c>
-      <c r="B31" s="7" t="s">
+      <c r="B45" s="7" t="s">
         <v>142</v>
-      </c>
-    </row>
-    <row r="32" spans="1:2" ht="45" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A32" s="12" t="s">
-        <v>112</v>
-      </c>
-      <c r="B32" s="11" t="s">
-        <v>143</v>
-      </c>
-    </row>
-    <row r="33" spans="1:2" ht="45" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A33" s="13" t="s">
-        <v>114</v>
-      </c>
-      <c r="B33" s="7" t="s">
-        <v>144</v>
-      </c>
-    </row>
-    <row r="34" spans="1:2" ht="45" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A34" s="12" t="s">
-        <v>116</v>
-      </c>
-      <c r="B34" s="11" t="s">
-        <v>145</v>
-      </c>
-    </row>
-    <row r="35" spans="1:2" ht="45" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A35" s="13" t="s">
-        <v>118</v>
-      </c>
-      <c r="B35" s="7" t="s">
-        <v>119</v>
-      </c>
-    </row>
-    <row r="36" spans="1:2" ht="45" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A36" s="12" t="s">
-        <v>120</v>
-      </c>
-      <c r="B36" s="11" t="s">
-        <v>119</v>
-      </c>
-    </row>
-    <row r="37" spans="1:2" ht="45" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A37" s="13" t="s">
-        <v>121</v>
-      </c>
-      <c r="B37" s="7" t="s">
-        <v>122</v>
-      </c>
-    </row>
-    <row r="38" spans="1:2" ht="45" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A38" s="12" t="s">
-        <v>123</v>
-      </c>
-      <c r="B38" s="11" t="s">
-        <v>146</v>
-      </c>
-    </row>
-    <row r="39" spans="1:2" ht="45" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A39" s="13" t="s">
-        <v>125</v>
-      </c>
-      <c r="B39" s="7" t="s">
-        <v>147</v>
-      </c>
-    </row>
-    <row r="40" spans="1:2" ht="45" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A40" s="12" t="s">
-        <v>127</v>
-      </c>
-      <c r="B40" s="11" t="s">
-        <v>119</v>
-      </c>
-    </row>
-    <row r="41" spans="1:2" ht="45" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A41" s="13" t="s">
-        <v>128</v>
-      </c>
-      <c r="B41" s="7" t="s">
-        <v>129</v>
-      </c>
-    </row>
-    <row r="42" spans="1:2" ht="45" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A42" s="12" t="s">
-        <v>130</v>
-      </c>
-      <c r="B42" s="11" t="s">
-        <v>142</v>
-      </c>
-    </row>
-    <row r="43" spans="1:2" ht="45" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A43" s="13" t="s">
-        <v>131</v>
-      </c>
-      <c r="B43" s="7" t="s">
-        <v>148</v>
-      </c>
-    </row>
-    <row r="44" spans="1:2" ht="45" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A44" s="12" t="s">
-        <v>133</v>
-      </c>
-      <c r="B44" s="11" t="s">
-        <v>134</v>
-      </c>
-    </row>
-    <row r="45" spans="1:2" ht="45" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A45" s="13" t="s">
-        <v>135</v>
-      </c>
-      <c r="B45" s="7" t="s">
-        <v>149</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Reapply "Add the Gateway and Diagnosis Validation"
This reverts commit edd536360d3516631d38d2ee44803e5500b67dc0.
</commit_message>
<xml_diff>
--- a/src/data/real_use_cases.xlsx
+++ b/src/data/real_use_cases.xlsx
@@ -9,7 +9,7 @@
     </mc:Choice>
   </mc:AlternateContent>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="28800" windowHeight="12300" activeTab="1"/>
+    <workbookView xWindow="0" yWindow="0" windowWidth="28800" windowHeight="12300"/>
   </bookViews>
   <sheets>
     <sheet name="Scripts" sheetId="1" r:id="rId1"/>
@@ -27,7 +27,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="255" uniqueCount="156">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="259" uniqueCount="158">
   <si>
     <t>Departement</t>
   </si>
@@ -118,6 +118,9 @@
     <t>Final Diagnosis</t>
   </si>
   <si>
+    <t>Unstable angina / acute coronary syndrome under evaluation.</t>
+  </si>
+  <si>
     <t>Plan of Care</t>
   </si>
   <si>
@@ -142,18 +145,33 @@
     <t>Expected</t>
   </si>
   <si>
+    <t>A – Airway</t>
+  </si>
+  <si>
     <t>Patent</t>
   </si>
   <si>
+    <t>B – Breathing</t>
+  </si>
+  <si>
     <t>Spontaneous breathing</t>
   </si>
   <si>
+    <t>C – Circulation</t>
+  </si>
+  <si>
     <t>Hemodynamically stabl</t>
   </si>
   <si>
+    <t>D – Disability</t>
+  </si>
+  <si>
     <t>No neurological abnormality reported</t>
   </si>
   <si>
+    <t>E – Exposure</t>
+  </si>
+  <si>
     <t>No significant abnormality reported.</t>
   </si>
   <si>
@@ -194,6 +212,9 @@
   </si>
   <si>
     <t>Patient is drowsy, pale, delirious, and has a disturbed conscious level. Laboratory findings showed anemia with hemoglobin 8.5 g/dL, elevated TLC, metabolic acidosis, and elevated renal function tests.</t>
+  </si>
+  <si>
+    <t>Acute confusional state with metabolic acidosis and renal impairment; possible acute kidney injury on top of chronic kidney disease, with sepsis/septic shock to be excluded.</t>
   </si>
   <si>
     <t>ICU admission. Close monitoring of conscious level, hemodynamic status, renal function, and acid-base status. Further infectious and metabolic workup. ICU consultant review. Infectious disease consultation for further evaluation and management.</t>
@@ -517,6 +538,22 @@
   </si>
   <si>
     <t>3 Months</t>
+  </si>
+  <si>
+    <r>
+      <t>Social / Marital / Family History</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t> </t>
+    </r>
+  </si>
+  <si>
+    <t>Plan of Care (short/long term)</t>
   </si>
   <si>
     <t>Procedures Planned</t>
@@ -551,37 +588,6 @@
 No internal referrals were required.  
 The patient will return after three months for healing assessment and prosthetic restoration planning.  
 Retention priority is high.</t>
-  </si>
-  <si>
-    <t>Airway</t>
-  </si>
-  <si>
-    <t>Breathing</t>
-  </si>
-  <si>
-    <t>Circulation</t>
-  </si>
-  <si>
-    <t>Disability</t>
-  </si>
-  <si>
-    <t>Exposure</t>
-  </si>
-  <si>
-    <t>Differential Diagnoses</t>
-  </si>
-  <si>
-    <r>
-      <t>Social Family History</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="12"/>
-        <rFont val="Arial"/>
-        <family val="2"/>
-      </rPr>
-      <t> </t>
-    </r>
   </si>
 </sst>
 </file>
@@ -794,7 +800,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="20">
+  <cellXfs count="21">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
@@ -815,6 +821,12 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="3" fillId="5" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="5" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="5" fillId="4" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
@@ -827,6 +839,12 @@
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
     <xf numFmtId="0" fontId="7" fillId="6" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
@@ -836,17 +854,8 @@
     <xf numFmtId="0" fontId="1" fillId="7" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="5" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="5" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
+    <xf numFmtId="0" fontId="0" fillId="7" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -1223,7 +1232,7 @@
         <v>4</v>
       </c>
       <c r="C9" s="5" t="s">
-        <v>148</v>
+        <v>157</v>
       </c>
     </row>
     <row r="10" spans="1:3" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
@@ -1282,52 +1291,52 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:B39"/>
+  <dimension ref="A1:B41"/>
   <sheetFormatPr defaultColWidth="22.140625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="2" max="2" width="79.28515625" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:2" ht="21" x14ac:dyDescent="0.25">
-      <c r="A1" s="15" t="s">
-        <v>40</v>
-      </c>
-      <c r="B1" s="16"/>
+      <c r="A1" s="8" t="s">
+        <v>46</v>
+      </c>
+      <c r="B1" s="9"/>
     </row>
     <row r="2" spans="1:2" ht="18.75" x14ac:dyDescent="0.25">
-      <c r="A2" s="8" t="s">
-        <v>32</v>
-      </c>
-      <c r="B2" s="8" t="s">
+      <c r="A2" s="10" t="s">
         <v>33</v>
       </c>
+      <c r="B2" s="10" t="s">
+        <v>34</v>
+      </c>
     </row>
     <row r="3" spans="1:2" ht="45" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A3" s="10" t="s">
+      <c r="A3" s="12" t="s">
         <v>12</v>
       </c>
-      <c r="B3" s="9" t="s">
+      <c r="B3" s="11" t="s">
         <v>13</v>
       </c>
     </row>
     <row r="4" spans="1:2" ht="45" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A4" s="11" t="s">
-        <v>154</v>
+      <c r="A4" s="13" t="s">
+        <v>45</v>
       </c>
       <c r="B4" s="6" t="s">
         <v>14</v>
       </c>
     </row>
     <row r="5" spans="1:2" ht="45" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A5" s="10" t="s">
+      <c r="A5" s="12" t="s">
         <v>15</v>
       </c>
-      <c r="B5" s="9" t="s">
+      <c r="B5" s="11" t="s">
         <v>16</v>
       </c>
     </row>
     <row r="6" spans="1:2" ht="45" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A6" s="11" t="s">
+      <c r="A6" s="13" t="s">
         <v>17</v>
       </c>
       <c r="B6" s="7" t="s">
@@ -1335,15 +1344,15 @@
       </c>
     </row>
     <row r="7" spans="1:2" ht="45" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A7" s="10" t="s">
+      <c r="A7" s="12" t="s">
         <v>18</v>
       </c>
-      <c r="B7" s="9" t="s">
+      <c r="B7" s="11" t="s">
         <v>16</v>
       </c>
     </row>
     <row r="8" spans="1:2" ht="45" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A8" s="11" t="s">
+      <c r="A8" s="13" t="s">
         <v>19</v>
       </c>
       <c r="B8" s="7" t="s">
@@ -1351,252 +1360,268 @@
       </c>
     </row>
     <row r="9" spans="1:2" ht="45" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A9" s="10" t="s">
+      <c r="A9" s="12" t="s">
         <v>21</v>
       </c>
-      <c r="B9" s="9" t="s">
+      <c r="B9" s="11" t="s">
         <v>22</v>
       </c>
     </row>
     <row r="10" spans="1:2" ht="45" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A10" s="12" t="s">
-        <v>149</v>
-      </c>
-      <c r="B10" s="13" t="s">
+      <c r="A10" s="16" t="s">
+        <v>35</v>
+      </c>
+      <c r="B10" s="17" t="s">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="11" spans="1:2" ht="45" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A11" s="12" t="s">
+        <v>37</v>
+      </c>
+      <c r="B11" s="11" t="s">
+        <v>38</v>
+      </c>
+    </row>
+    <row r="12" spans="1:2" ht="45" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A12" s="16" t="s">
+        <v>39</v>
+      </c>
+      <c r="B12" s="17" t="s">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="13" spans="1:2" ht="45" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A13" s="12" t="s">
+        <v>41</v>
+      </c>
+      <c r="B13" s="11" t="s">
+        <v>42</v>
+      </c>
+    </row>
+    <row r="14" spans="1:2" ht="45" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A14" s="16" t="s">
+        <v>43</v>
+      </c>
+      <c r="B14" s="17" t="s">
+        <v>44</v>
+      </c>
+    </row>
+    <row r="15" spans="1:2" ht="45" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A15" s="12" t="s">
+        <v>23</v>
+      </c>
+      <c r="B15" s="11" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="16" spans="1:2" ht="45" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A16" s="16" t="s">
+        <v>25</v>
+      </c>
+      <c r="B16" s="17" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="17" spans="1:2" ht="45" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A17" s="12" t="s">
+        <v>27</v>
+      </c>
+      <c r="B17" s="11" t="s">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="18" spans="1:2" ht="45" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A18" s="16" t="s">
+        <v>29</v>
+      </c>
+      <c r="B18" s="17" t="s">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="19" spans="1:2" ht="45" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A19" s="12" t="s">
+        <v>31</v>
+      </c>
+      <c r="B19" s="11" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="20" spans="1:2" ht="45" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A20" s="18" t="s">
+        <v>48</v>
+      </c>
+      <c r="B20" s="19" t="s">
+        <v>49</v>
+      </c>
+    </row>
+    <row r="21" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A21" s="14"/>
+      <c r="B21" s="14"/>
+    </row>
+    <row r="22" spans="1:2" ht="21" x14ac:dyDescent="0.25">
+      <c r="A22" s="8" t="s">
+        <v>47</v>
+      </c>
+      <c r="B22" s="9"/>
+    </row>
+    <row r="23" spans="1:2" ht="18.75" x14ac:dyDescent="0.25">
+      <c r="A23" s="10" t="s">
+        <v>33</v>
+      </c>
+      <c r="B23" s="10" t="s">
         <v>34</v>
       </c>
     </row>
-    <row r="11" spans="1:2" ht="45" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A11" s="10" t="s">
-        <v>150</v>
-      </c>
-      <c r="B11" s="9" t="s">
-        <v>35</v>
-      </c>
-    </row>
-    <row r="12" spans="1:2" ht="45" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A12" s="12" t="s">
-        <v>151</v>
-      </c>
-      <c r="B12" s="13" t="s">
-        <v>36</v>
-      </c>
-    </row>
-    <row r="13" spans="1:2" ht="45" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A13" s="10" t="s">
-        <v>152</v>
-      </c>
-      <c r="B13" s="9" t="s">
-        <v>37</v>
-      </c>
-    </row>
-    <row r="14" spans="1:2" ht="45" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A14" s="12" t="s">
-        <v>153</v>
-      </c>
-      <c r="B14" s="13" t="s">
-        <v>38</v>
-      </c>
-    </row>
-    <row r="15" spans="1:2" ht="45" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A15" s="10" t="s">
-        <v>23</v>
-      </c>
-      <c r="B15" s="9" t="s">
-        <v>24</v>
-      </c>
-    </row>
-    <row r="16" spans="1:2" ht="45" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A16" s="12" t="s">
-        <v>26</v>
-      </c>
-      <c r="B16" s="12" t="s">
-        <v>27</v>
-      </c>
-    </row>
-    <row r="17" spans="1:2" ht="45" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A17" s="10" t="s">
-        <v>28</v>
-      </c>
-      <c r="B17" s="10" t="s">
-        <v>29</v>
-      </c>
-    </row>
-    <row r="18" spans="1:2" ht="45" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A18" s="14" t="s">
-        <v>30</v>
-      </c>
-      <c r="B18" s="14" t="s">
-        <v>31</v>
-      </c>
-    </row>
-    <row r="19" spans="1:2" ht="45" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A19" s="10" t="s">
-        <v>42</v>
-      </c>
-      <c r="B19" s="10" t="s">
-        <v>43</v>
-      </c>
-    </row>
-    <row r="20" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A20" s="17"/>
-      <c r="B20" s="17"/>
-    </row>
-    <row r="21" spans="1:2" ht="21" x14ac:dyDescent="0.25">
-      <c r="A21" s="15" t="s">
-        <v>41</v>
-      </c>
-      <c r="B21" s="16"/>
-    </row>
-    <row r="22" spans="1:2" ht="18.75" x14ac:dyDescent="0.25">
-      <c r="A22" s="8" t="s">
-        <v>32</v>
-      </c>
-      <c r="B22" s="8" t="s">
-        <v>33</v>
-      </c>
-    </row>
-    <row r="23" spans="1:2" ht="48" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A23" s="11" t="s">
+    <row r="24" spans="1:2" ht="48" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A24" s="13" t="s">
         <v>12</v>
       </c>
-      <c r="B23" s="1" t="s">
-        <v>44</v>
-      </c>
-    </row>
-    <row r="24" spans="1:2" ht="48" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A24" s="10" t="s">
-        <v>154</v>
-      </c>
-      <c r="B24" s="9" t="s">
+      <c r="B24" s="1" t="s">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="25" spans="1:2" ht="48" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A25" s="12" t="s">
         <v>45</v>
       </c>
-    </row>
-    <row r="25" spans="1:2" ht="48" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A25" s="11" t="s">
+      <c r="B25" s="11" t="s">
+        <v>51</v>
+      </c>
+    </row>
+    <row r="26" spans="1:2" ht="48" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A26" s="13" t="s">
         <v>15</v>
       </c>
-      <c r="B25" s="1" t="s">
-        <v>46</v>
-      </c>
-    </row>
-    <row r="26" spans="1:2" ht="48" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A26" s="10" t="s">
+      <c r="B26" s="1" t="s">
+        <v>52</v>
+      </c>
+    </row>
+    <row r="27" spans="1:2" ht="48" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A27" s="12" t="s">
         <v>17</v>
       </c>
-      <c r="B26" s="9" t="s">
-        <v>47</v>
-      </c>
-    </row>
-    <row r="27" spans="1:2" ht="48" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A27" s="11" t="s">
+      <c r="B27" s="11" t="s">
+        <v>53</v>
+      </c>
+    </row>
+    <row r="28" spans="1:2" ht="48" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A28" s="13" t="s">
         <v>18</v>
       </c>
-      <c r="B27" s="1" t="s">
-        <v>48</v>
-      </c>
-    </row>
-    <row r="28" spans="1:2" ht="48" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A28" s="10" t="s">
+      <c r="B28" s="1" t="s">
+        <v>54</v>
+      </c>
+    </row>
+    <row r="29" spans="1:2" ht="48" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A29" s="12" t="s">
         <v>19</v>
       </c>
-      <c r="B28" s="9" t="s">
-        <v>49</v>
-      </c>
-    </row>
-    <row r="29" spans="1:2" ht="48" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A29" s="11" t="s">
+      <c r="B29" s="11" t="s">
+        <v>55</v>
+      </c>
+    </row>
+    <row r="30" spans="1:2" ht="48" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A30" s="13" t="s">
         <v>21</v>
       </c>
-      <c r="B29" s="1" t="s">
-        <v>50</v>
-      </c>
-    </row>
-    <row r="30" spans="1:2" ht="48" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A30" s="10" t="s">
-        <v>149</v>
-      </c>
-      <c r="B30" s="9" t="s">
-        <v>34</v>
+      <c r="B30" s="1" t="s">
+        <v>56</v>
       </c>
     </row>
     <row r="31" spans="1:2" ht="48" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A31" s="12" t="s">
-        <v>150</v>
-      </c>
-      <c r="B31" s="13" t="s">
-        <v>55</v>
+        <v>35</v>
+      </c>
+      <c r="B31" s="11" t="s">
+        <v>36</v>
       </c>
     </row>
     <row r="32" spans="1:2" ht="48" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A32" s="10" t="s">
-        <v>151</v>
-      </c>
-      <c r="B32" s="9" t="s">
-        <v>56</v>
+      <c r="A32" s="16" t="s">
+        <v>37</v>
+      </c>
+      <c r="B32" s="17" t="s">
+        <v>62</v>
       </c>
     </row>
     <row r="33" spans="1:2" ht="48" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A33" s="12" t="s">
-        <v>152</v>
-      </c>
-      <c r="B33" s="13" t="s">
-        <v>57</v>
+        <v>39</v>
+      </c>
+      <c r="B33" s="11" t="s">
+        <v>63</v>
       </c>
     </row>
     <row r="34" spans="1:2" ht="48" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A34" s="10" t="s">
-        <v>153</v>
-      </c>
-      <c r="B34" s="9" t="s">
-        <v>58</v>
+      <c r="A34" s="16" t="s">
+        <v>41</v>
+      </c>
+      <c r="B34" s="17" t="s">
+        <v>64</v>
       </c>
     </row>
     <row r="35" spans="1:2" ht="48" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A35" s="12" t="s">
+        <v>43</v>
+      </c>
+      <c r="B35" s="11" t="s">
+        <v>65</v>
+      </c>
+    </row>
+    <row r="36" spans="1:2" ht="48" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A36" s="16" t="s">
         <v>23</v>
       </c>
-      <c r="B35" s="13" t="s">
-        <v>51</v>
-      </c>
-    </row>
-    <row r="36" spans="1:2" ht="48" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A36" s="10" t="s">
-        <v>26</v>
-      </c>
-      <c r="B36" s="9" t="s">
-        <v>52</v>
+      <c r="B36" s="17" t="s">
+        <v>57</v>
       </c>
     </row>
     <row r="37" spans="1:2" ht="48" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A37" s="12" t="s">
-        <v>28</v>
-      </c>
-      <c r="B37" s="12" t="s">
-        <v>53</v>
+        <v>25</v>
+      </c>
+      <c r="B37" s="11" t="s">
+        <v>58</v>
       </c>
     </row>
     <row r="38" spans="1:2" ht="48" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A38" s="10" t="s">
-        <v>30</v>
-      </c>
-      <c r="B38" s="10" t="s">
-        <v>54</v>
+      <c r="A38" s="16" t="s">
+        <v>27</v>
+      </c>
+      <c r="B38" s="17" t="s">
+        <v>59</v>
       </c>
     </row>
     <row r="39" spans="1:2" ht="48" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A39" s="12" t="s">
-        <v>42</v>
-      </c>
-      <c r="B39" s="12" t="s">
-        <v>43</v>
+        <v>29</v>
+      </c>
+      <c r="B39" s="11" t="s">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="40" spans="1:2" ht="48" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A40" s="16" t="s">
+        <v>31</v>
+      </c>
+      <c r="B40" s="17" t="s">
+        <v>61</v>
+      </c>
+    </row>
+    <row r="41" spans="1:2" ht="48" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A41" s="12" t="s">
+        <v>48</v>
+      </c>
+      <c r="B41" s="11" t="s">
+        <v>49</v>
       </c>
     </row>
   </sheetData>
   <mergeCells count="3">
     <mergeCell ref="A1:B1"/>
+    <mergeCell ref="A22:B22"/>
     <mergeCell ref="A21:B21"/>
-    <mergeCell ref="A20:B20"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" r:id="rId1"/>
@@ -1612,307 +1637,307 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:2" ht="21" x14ac:dyDescent="0.25">
-      <c r="A1" s="15" t="s">
+      <c r="A1" s="8" t="s">
+        <v>85</v>
+      </c>
+      <c r="B1" s="9"/>
+    </row>
+    <row r="2" spans="1:2" ht="18.75" x14ac:dyDescent="0.25">
+      <c r="A2" s="10" t="s">
+        <v>33</v>
+      </c>
+      <c r="B2" s="10" t="s">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="3" spans="1:2" ht="45" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A3" s="12" t="s">
+        <v>12</v>
+      </c>
+      <c r="B3" s="11" t="s">
+        <v>66</v>
+      </c>
+    </row>
+    <row r="4" spans="1:2" ht="45" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A4" s="13" t="s">
+        <v>15</v>
+      </c>
+      <c r="B4" s="7" t="s">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="5" spans="1:2" ht="45" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A5" s="12" t="s">
+        <v>17</v>
+      </c>
+      <c r="B5" s="11" t="s">
+        <v>98</v>
+      </c>
+    </row>
+    <row r="6" spans="1:2" ht="45" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A6" s="13" t="s">
+        <v>18</v>
+      </c>
+      <c r="B6" s="7" t="s">
+        <v>99</v>
+      </c>
+    </row>
+    <row r="7" spans="1:2" ht="45" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A7" s="12" t="s">
+        <v>67</v>
+      </c>
+      <c r="B7" s="11" t="s">
+        <v>68</v>
+      </c>
+    </row>
+    <row r="8" spans="1:2" ht="45" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A8" s="13" t="s">
+        <v>97</v>
+      </c>
+      <c r="B8" s="7" t="s">
+        <v>69</v>
+      </c>
+    </row>
+    <row r="9" spans="1:2" ht="45" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A9" s="12" t="s">
+        <v>70</v>
+      </c>
+      <c r="B9" s="11" t="s">
+        <v>71</v>
+      </c>
+    </row>
+    <row r="10" spans="1:2" ht="45" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A10" s="13" t="s">
+        <v>72</v>
+      </c>
+      <c r="B10" s="7" t="s">
+        <v>73</v>
+      </c>
+    </row>
+    <row r="11" spans="1:2" ht="45" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A11" s="12" t="s">
+        <v>150</v>
+      </c>
+      <c r="B11" s="11" t="s">
+        <v>74</v>
+      </c>
+    </row>
+    <row r="12" spans="1:2" ht="45" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A12" s="13" t="s">
+        <v>155</v>
+      </c>
+      <c r="B12" s="7" t="s">
+        <v>75</v>
+      </c>
+    </row>
+    <row r="13" spans="1:2" ht="45" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A13" s="12" t="s">
+        <v>151</v>
+      </c>
+      <c r="B13" s="11" t="s">
+        <v>76</v>
+      </c>
+    </row>
+    <row r="14" spans="1:2" ht="45" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A14" s="13" t="s">
+        <v>152</v>
+      </c>
+      <c r="B14" s="7" t="s">
+        <v>77</v>
+      </c>
+    </row>
+    <row r="15" spans="1:2" ht="45" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A15" s="12" t="s">
         <v>78</v>
       </c>
-      <c r="B1" s="16"/>
-    </row>
-    <row r="2" spans="1:2" ht="18.75" x14ac:dyDescent="0.25">
-      <c r="A2" s="8" t="s">
-        <v>32</v>
-      </c>
-      <c r="B2" s="8" t="s">
+      <c r="B15" s="11" t="s">
+        <v>79</v>
+      </c>
+    </row>
+    <row r="16" spans="1:2" ht="45" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A16" s="13" t="s">
+        <v>153</v>
+      </c>
+      <c r="B16" s="7" t="s">
+        <v>80</v>
+      </c>
+    </row>
+    <row r="17" spans="1:2" ht="45" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A17" s="12" t="s">
+        <v>81</v>
+      </c>
+      <c r="B17" s="11" t="s">
+        <v>82</v>
+      </c>
+    </row>
+    <row r="18" spans="1:2" ht="45" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A18" s="13" t="s">
+        <v>156</v>
+      </c>
+      <c r="B18" s="7" t="s">
+        <v>83</v>
+      </c>
+    </row>
+    <row r="19" spans="1:2" ht="45" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A19" s="12" t="s">
+        <v>154</v>
+      </c>
+      <c r="B19" s="11" t="s">
+        <v>84</v>
+      </c>
+    </row>
+    <row r="20" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A20" s="15"/>
+      <c r="B20" s="15"/>
+    </row>
+    <row r="21" spans="1:2" ht="21" x14ac:dyDescent="0.25">
+      <c r="A21" s="8" t="s">
+        <v>86</v>
+      </c>
+      <c r="B21" s="9"/>
+    </row>
+    <row r="22" spans="1:2" ht="18.75" x14ac:dyDescent="0.25">
+      <c r="A22" s="10" t="s">
         <v>33</v>
       </c>
-    </row>
-    <row r="3" spans="1:2" ht="45" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A3" s="10" t="s">
+      <c r="B22" s="10" t="s">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="23" spans="1:2" ht="45" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A23" s="12" t="s">
         <v>12</v>
       </c>
-      <c r="B3" s="9" t="s">
-        <v>59</v>
-      </c>
-    </row>
-    <row r="4" spans="1:2" ht="45" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A4" s="11" t="s">
+      <c r="B23" s="11" t="s">
+        <v>87</v>
+      </c>
+    </row>
+    <row r="24" spans="1:2" ht="45" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A24" s="13" t="s">
         <v>15</v>
       </c>
-      <c r="B4" s="7" t="s">
+      <c r="B24" s="7" t="s">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="25" spans="1:2" ht="45" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A25" s="12" t="s">
+        <v>17</v>
+      </c>
+      <c r="B25" s="11" t="s">
+        <v>98</v>
+      </c>
+    </row>
+    <row r="26" spans="1:2" ht="45" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A26" s="13" t="s">
+        <v>18</v>
+      </c>
+      <c r="B26" s="7" t="s">
+        <v>101</v>
+      </c>
+    </row>
+    <row r="27" spans="1:2" ht="45" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A27" s="12" t="s">
+        <v>67</v>
+      </c>
+      <c r="B27" s="11" t="s">
+        <v>68</v>
+      </c>
+    </row>
+    <row r="28" spans="1:2" ht="45" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A28" s="13" t="s">
+        <v>97</v>
+      </c>
+      <c r="B28" s="17" t="s">
+        <v>88</v>
+      </c>
+    </row>
+    <row r="29" spans="1:2" ht="45" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A29" s="12" t="s">
+        <v>70</v>
+      </c>
+      <c r="B29" s="11" t="s">
+        <v>89</v>
+      </c>
+    </row>
+    <row r="30" spans="1:2" ht="45" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A30" s="13" t="s">
+        <v>72</v>
+      </c>
+      <c r="B30" s="17" t="s">
+        <v>73</v>
+      </c>
+    </row>
+    <row r="31" spans="1:2" ht="45" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A31" s="12" t="s">
+        <v>150</v>
+      </c>
+      <c r="B31" s="11" t="s">
+        <v>90</v>
+      </c>
+    </row>
+    <row r="32" spans="1:2" ht="45" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A32" s="13" t="s">
+        <v>155</v>
+      </c>
+      <c r="B32" s="17" t="s">
+        <v>91</v>
+      </c>
+    </row>
+    <row r="33" spans="1:2" ht="45" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A33" s="12" t="s">
+        <v>151</v>
+      </c>
+      <c r="B33" s="11" t="s">
+        <v>92</v>
+      </c>
+    </row>
+    <row r="34" spans="1:2" ht="45" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A34" s="13" t="s">
+        <v>152</v>
+      </c>
+      <c r="B34" s="17" t="s">
         <v>93</v>
       </c>
     </row>
-    <row r="5" spans="1:2" ht="45" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A5" s="10" t="s">
-        <v>17</v>
-      </c>
-      <c r="B5" s="9" t="s">
-        <v>91</v>
-      </c>
-    </row>
-    <row r="6" spans="1:2" ht="45" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A6" s="11" t="s">
-        <v>18</v>
-      </c>
-      <c r="B6" s="7" t="s">
-        <v>92</v>
-      </c>
-    </row>
-    <row r="7" spans="1:2" ht="45" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A7" s="10" t="s">
-        <v>60</v>
-      </c>
-      <c r="B7" s="9" t="s">
-        <v>61</v>
-      </c>
-    </row>
-    <row r="8" spans="1:2" ht="45" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A8" s="11" t="s">
-        <v>90</v>
-      </c>
-      <c r="B8" s="7" t="s">
-        <v>62</v>
-      </c>
-    </row>
-    <row r="9" spans="1:2" ht="45" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A9" s="10" t="s">
-        <v>63</v>
-      </c>
-      <c r="B9" s="9" t="s">
-        <v>64</v>
-      </c>
-    </row>
-    <row r="10" spans="1:2" ht="45" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A10" s="11" t="s">
-        <v>65</v>
-      </c>
-      <c r="B10" s="7" t="s">
-        <v>66</v>
-      </c>
-    </row>
-    <row r="11" spans="1:2" ht="45" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A11" s="10" t="s">
-        <v>155</v>
-      </c>
-      <c r="B11" s="9" t="s">
-        <v>67</v>
-      </c>
-    </row>
-    <row r="12" spans="1:2" ht="45" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A12" s="11" t="s">
-        <v>146</v>
-      </c>
-      <c r="B12" s="7" t="s">
-        <v>68</v>
-      </c>
-    </row>
-    <row r="13" spans="1:2" ht="45" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A13" s="10" t="s">
-        <v>26</v>
-      </c>
-      <c r="B13" s="9" t="s">
-        <v>69</v>
-      </c>
-    </row>
-    <row r="14" spans="1:2" ht="45" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A14" s="11" t="s">
-        <v>143</v>
-      </c>
-      <c r="B14" s="7" t="s">
-        <v>70</v>
-      </c>
-    </row>
-    <row r="15" spans="1:2" ht="45" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A15" s="10" t="s">
-        <v>71</v>
-      </c>
-      <c r="B15" s="9" t="s">
-        <v>72</v>
-      </c>
-    </row>
-    <row r="16" spans="1:2" ht="45" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A16" s="11" t="s">
-        <v>144</v>
-      </c>
-      <c r="B16" s="7" t="s">
-        <v>73</v>
-      </c>
-    </row>
-    <row r="17" spans="1:2" ht="45" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A17" s="10" t="s">
-        <v>74</v>
-      </c>
-      <c r="B17" s="9" t="s">
-        <v>75</v>
-      </c>
-    </row>
-    <row r="18" spans="1:2" ht="45" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A18" s="11" t="s">
-        <v>147</v>
-      </c>
-      <c r="B18" s="7" t="s">
-        <v>76</v>
-      </c>
-    </row>
-    <row r="19" spans="1:2" ht="45" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A19" s="10" t="s">
-        <v>145</v>
-      </c>
-      <c r="B19" s="9" t="s">
-        <v>77</v>
-      </c>
-    </row>
-    <row r="20" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A20" s="18"/>
-      <c r="B20" s="18"/>
-    </row>
-    <row r="21" spans="1:2" ht="21" x14ac:dyDescent="0.25">
-      <c r="A21" s="15" t="s">
-        <v>79</v>
-      </c>
-      <c r="B21" s="16"/>
-    </row>
-    <row r="22" spans="1:2" ht="18.75" x14ac:dyDescent="0.25">
-      <c r="A22" s="8" t="s">
-        <v>32</v>
-      </c>
-      <c r="B22" s="8" t="s">
-        <v>33</v>
-      </c>
-    </row>
-    <row r="23" spans="1:2" ht="45" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A23" s="10" t="s">
-        <v>12</v>
-      </c>
-      <c r="B23" s="9" t="s">
-        <v>80</v>
-      </c>
-    </row>
-    <row r="24" spans="1:2" ht="45" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A24" s="11" t="s">
-        <v>15</v>
-      </c>
-      <c r="B24" s="7" t="s">
-        <v>93</v>
-      </c>
-    </row>
-    <row r="25" spans="1:2" ht="45" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A25" s="10" t="s">
-        <v>17</v>
-      </c>
-      <c r="B25" s="9" t="s">
-        <v>91</v>
-      </c>
-    </row>
-    <row r="26" spans="1:2" ht="45" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A26" s="11" t="s">
-        <v>18</v>
-      </c>
-      <c r="B26" s="7" t="s">
+    <row r="35" spans="1:2" ht="45" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A35" s="12" t="s">
+        <v>78</v>
+      </c>
+      <c r="B35" s="11" t="s">
         <v>94</v>
       </c>
     </row>
-    <row r="27" spans="1:2" ht="45" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A27" s="10" t="s">
-        <v>60</v>
-      </c>
-      <c r="B27" s="9" t="s">
-        <v>61</v>
-      </c>
-    </row>
-    <row r="28" spans="1:2" ht="45" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A28" s="11" t="s">
-        <v>90</v>
-      </c>
-      <c r="B28" s="13" t="s">
+    <row r="36" spans="1:2" ht="45" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A36" s="13" t="s">
+        <v>153</v>
+      </c>
+      <c r="B36" s="17" t="s">
+        <v>95</v>
+      </c>
+    </row>
+    <row r="37" spans="1:2" ht="45" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A37" s="12" t="s">
         <v>81</v>
       </c>
-    </row>
-    <row r="29" spans="1:2" ht="45" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A29" s="10" t="s">
-        <v>63</v>
-      </c>
-      <c r="B29" s="9" t="s">
-        <v>82</v>
-      </c>
-    </row>
-    <row r="30" spans="1:2" ht="45" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A30" s="11" t="s">
-        <v>65</v>
-      </c>
-      <c r="B30" s="13" t="s">
-        <v>66</v>
-      </c>
-    </row>
-    <row r="31" spans="1:2" ht="45" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A31" s="10" t="s">
-        <v>155</v>
-      </c>
-      <c r="B31" s="9" t="s">
+      <c r="B37" s="11" t="s">
+        <v>96</v>
+      </c>
+    </row>
+    <row r="38" spans="1:2" ht="45" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A38" s="13" t="s">
+        <v>156</v>
+      </c>
+      <c r="B38" s="17" t="s">
         <v>83</v>
       </c>
     </row>
-    <row r="32" spans="1:2" ht="45" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A32" s="11" t="s">
-        <v>146</v>
-      </c>
-      <c r="B32" s="13" t="s">
+    <row r="39" spans="1:2" ht="45" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A39" s="12" t="s">
+        <v>154</v>
+      </c>
+      <c r="B39" s="11" t="s">
         <v>84</v>
-      </c>
-    </row>
-    <row r="33" spans="1:2" ht="45" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A33" s="10" t="s">
-        <v>26</v>
-      </c>
-      <c r="B33" s="9" t="s">
-        <v>85</v>
-      </c>
-    </row>
-    <row r="34" spans="1:2" ht="45" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A34" s="11" t="s">
-        <v>143</v>
-      </c>
-      <c r="B34" s="13" t="s">
-        <v>86</v>
-      </c>
-    </row>
-    <row r="35" spans="1:2" ht="45" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A35" s="10" t="s">
-        <v>71</v>
-      </c>
-      <c r="B35" s="9" t="s">
-        <v>87</v>
-      </c>
-    </row>
-    <row r="36" spans="1:2" ht="45" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A36" s="11" t="s">
-        <v>144</v>
-      </c>
-      <c r="B36" s="13" t="s">
-        <v>88</v>
-      </c>
-    </row>
-    <row r="37" spans="1:2" ht="45" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A37" s="10" t="s">
-        <v>74</v>
-      </c>
-      <c r="B37" s="9" t="s">
-        <v>89</v>
-      </c>
-    </row>
-    <row r="38" spans="1:2" ht="45" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A38" s="11" t="s">
-        <v>147</v>
-      </c>
-      <c r="B38" s="13" t="s">
-        <v>76</v>
-      </c>
-    </row>
-    <row r="39" spans="1:2" ht="45" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A39" s="10" t="s">
-        <v>145</v>
-      </c>
-      <c r="B39" s="9" t="s">
-        <v>77</v>
       </c>
     </row>
   </sheetData>
@@ -1936,355 +1961,355 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:2" ht="21" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="15" t="s">
-        <v>95</v>
-      </c>
-      <c r="B1" s="16"/>
+      <c r="A1" s="8" t="s">
+        <v>102</v>
+      </c>
+      <c r="B1" s="9"/>
     </row>
     <row r="2" spans="1:2" ht="18.75" x14ac:dyDescent="0.25">
-      <c r="A2" s="8" t="s">
-        <v>32</v>
-      </c>
-      <c r="B2" s="8" t="s">
+      <c r="A2" s="10" t="s">
         <v>33</v>
       </c>
+      <c r="B2" s="10" t="s">
+        <v>34</v>
+      </c>
     </row>
     <row r="3" spans="1:2" ht="45" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A3" s="10" t="s">
-        <v>96</v>
-      </c>
-      <c r="B3" s="9" t="s">
-        <v>97</v>
+      <c r="A3" s="12" t="s">
+        <v>103</v>
+      </c>
+      <c r="B3" s="11" t="s">
+        <v>104</v>
       </c>
     </row>
     <row r="4" spans="1:2" ht="45" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A4" s="11" t="s">
-        <v>98</v>
+      <c r="A4" s="13" t="s">
+        <v>105</v>
       </c>
       <c r="B4" s="7" t="s">
-        <v>99</v>
+        <v>106</v>
       </c>
     </row>
     <row r="5" spans="1:2" ht="45" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A5" s="10" t="s">
+      <c r="A5" s="12" t="s">
         <v>12</v>
       </c>
-      <c r="B5" s="9" t="s">
-        <v>100</v>
+      <c r="B5" s="11" t="s">
+        <v>107</v>
       </c>
     </row>
     <row r="6" spans="1:2" ht="45" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A6" s="11" t="s">
-        <v>39</v>
+      <c r="A6" s="13" t="s">
+        <v>45</v>
       </c>
       <c r="B6" s="7" t="s">
-        <v>101</v>
+        <v>108</v>
       </c>
     </row>
     <row r="7" spans="1:2" ht="45" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A7" s="10" t="s">
+      <c r="A7" s="12" t="s">
         <v>25</v>
       </c>
-      <c r="B7" s="9" t="s">
-        <v>102</v>
+      <c r="B7" s="11" t="s">
+        <v>109</v>
       </c>
     </row>
     <row r="8" spans="1:2" ht="45" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A8" s="11" t="s">
+      <c r="A8" s="13" t="s">
+        <v>110</v>
+      </c>
+      <c r="B8" s="7" t="s">
+        <v>111</v>
+      </c>
+    </row>
+    <row r="9" spans="1:2" ht="45" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A9" s="12" t="s">
+        <v>112</v>
+      </c>
+      <c r="B9" s="11" t="s">
+        <v>113</v>
+      </c>
+    </row>
+    <row r="10" spans="1:2" ht="45" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A10" s="13" t="s">
+        <v>114</v>
+      </c>
+      <c r="B10" s="7" t="s">
+        <v>115</v>
+      </c>
+    </row>
+    <row r="11" spans="1:2" ht="45" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A11" s="12" t="s">
+        <v>116</v>
+      </c>
+      <c r="B11" s="11" t="s">
+        <v>117</v>
+      </c>
+    </row>
+    <row r="12" spans="1:2" ht="45" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A12" s="13" t="s">
+        <v>118</v>
+      </c>
+      <c r="B12" s="7" t="s">
+        <v>119</v>
+      </c>
+    </row>
+    <row r="13" spans="1:2" ht="45" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A13" s="12" t="s">
+        <v>120</v>
+      </c>
+      <c r="B13" s="11" t="s">
+        <v>119</v>
+      </c>
+    </row>
+    <row r="14" spans="1:2" ht="45" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A14" s="13" t="s">
+        <v>121</v>
+      </c>
+      <c r="B14" s="7" t="s">
+        <v>122</v>
+      </c>
+    </row>
+    <row r="15" spans="1:2" ht="45" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A15" s="12" t="s">
+        <v>123</v>
+      </c>
+      <c r="B15" s="11" t="s">
+        <v>124</v>
+      </c>
+    </row>
+    <row r="16" spans="1:2" ht="45" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A16" s="13" t="s">
+        <v>125</v>
+      </c>
+      <c r="B16" s="7" t="s">
+        <v>126</v>
+      </c>
+    </row>
+    <row r="17" spans="1:2" ht="45" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A17" s="12" t="s">
+        <v>127</v>
+      </c>
+      <c r="B17" s="11" t="s">
+        <v>122</v>
+      </c>
+    </row>
+    <row r="18" spans="1:2" ht="45" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A18" s="16" t="s">
+        <v>128</v>
+      </c>
+      <c r="B18" s="17" t="s">
+        <v>129</v>
+      </c>
+    </row>
+    <row r="19" spans="1:2" ht="45" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A19" s="12" t="s">
+        <v>130</v>
+      </c>
+      <c r="B19" s="11" t="s">
+        <v>111</v>
+      </c>
+    </row>
+    <row r="20" spans="1:2" ht="45" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A20" s="16" t="s">
+        <v>131</v>
+      </c>
+      <c r="B20" s="17" t="s">
+        <v>132</v>
+      </c>
+    </row>
+    <row r="21" spans="1:2" ht="45" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A21" s="12" t="s">
+        <v>133</v>
+      </c>
+      <c r="B21" s="11" t="s">
+        <v>134</v>
+      </c>
+    </row>
+    <row r="22" spans="1:2" ht="45" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A22" s="16" t="s">
+        <v>135</v>
+      </c>
+      <c r="B22" s="17" t="s">
+        <v>136</v>
+      </c>
+    </row>
+    <row r="23" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A23" s="20"/>
+      <c r="B23" s="20"/>
+    </row>
+    <row r="24" spans="1:2" ht="21" x14ac:dyDescent="0.25">
+      <c r="A24" s="8" t="s">
+        <v>137</v>
+      </c>
+      <c r="B24" s="9"/>
+    </row>
+    <row r="25" spans="1:2" ht="18.75" x14ac:dyDescent="0.25">
+      <c r="A25" s="10" t="s">
+        <v>33</v>
+      </c>
+      <c r="B25" s="10" t="s">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="26" spans="1:2" ht="45" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A26" s="12" t="s">
         <v>103</v>
       </c>
-      <c r="B8" s="7" t="s">
-        <v>104</v>
-      </c>
-    </row>
-    <row r="9" spans="1:2" ht="45" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A9" s="10" t="s">
+      <c r="B26" s="11" t="s">
+        <v>122</v>
+      </c>
+    </row>
+    <row r="27" spans="1:2" ht="45" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A27" s="13" t="s">
         <v>105</v>
       </c>
-      <c r="B9" s="9" t="s">
-        <v>106</v>
-      </c>
-    </row>
-    <row r="10" spans="1:2" ht="45" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A10" s="11" t="s">
-        <v>107</v>
-      </c>
-      <c r="B10" s="7" t="s">
-        <v>108</v>
-      </c>
-    </row>
-    <row r="11" spans="1:2" ht="45" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A11" s="10" t="s">
-        <v>109</v>
-      </c>
-      <c r="B11" s="9" t="s">
+      <c r="B27" s="7" t="s">
+        <v>138</v>
+      </c>
+    </row>
+    <row r="28" spans="1:2" ht="45" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A28" s="12" t="s">
+        <v>12</v>
+      </c>
+      <c r="B28" s="11" t="s">
+        <v>139</v>
+      </c>
+    </row>
+    <row r="29" spans="1:2" ht="45" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A29" s="13" t="s">
+        <v>45</v>
+      </c>
+      <c r="B29" s="7" t="s">
+        <v>140</v>
+      </c>
+    </row>
+    <row r="30" spans="1:2" ht="45" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A30" s="12" t="s">
+        <v>25</v>
+      </c>
+      <c r="B30" s="11" t="s">
+        <v>141</v>
+      </c>
+    </row>
+    <row r="31" spans="1:2" ht="45" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A31" s="13" t="s">
         <v>110</v>
       </c>
-    </row>
-    <row r="12" spans="1:2" ht="45" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A12" s="11" t="s">
-        <v>111</v>
-      </c>
-      <c r="B12" s="7" t="s">
+      <c r="B31" s="7" t="s">
+        <v>142</v>
+      </c>
+    </row>
+    <row r="32" spans="1:2" ht="45" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A32" s="12" t="s">
         <v>112</v>
       </c>
-    </row>
-    <row r="13" spans="1:2" ht="45" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A13" s="10" t="s">
-        <v>113</v>
-      </c>
-      <c r="B13" s="9" t="s">
-        <v>112</v>
-      </c>
-    </row>
-    <row r="14" spans="1:2" ht="45" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A14" s="11" t="s">
+      <c r="B32" s="11" t="s">
+        <v>143</v>
+      </c>
+    </row>
+    <row r="33" spans="1:2" ht="45" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A33" s="13" t="s">
         <v>114</v>
       </c>
-      <c r="B14" s="7" t="s">
-        <v>115</v>
-      </c>
-    </row>
-    <row r="15" spans="1:2" ht="45" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A15" s="10" t="s">
+      <c r="B33" s="7" t="s">
+        <v>144</v>
+      </c>
+    </row>
+    <row r="34" spans="1:2" ht="45" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A34" s="12" t="s">
         <v>116</v>
       </c>
-      <c r="B15" s="9" t="s">
-        <v>117</v>
-      </c>
-    </row>
-    <row r="16" spans="1:2" ht="45" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A16" s="11" t="s">
+      <c r="B34" s="11" t="s">
+        <v>145</v>
+      </c>
+    </row>
+    <row r="35" spans="1:2" ht="45" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A35" s="13" t="s">
         <v>118</v>
       </c>
-      <c r="B16" s="7" t="s">
+      <c r="B35" s="7" t="s">
         <v>119</v>
       </c>
     </row>
-    <row r="17" spans="1:2" ht="45" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A17" s="10" t="s">
+    <row r="36" spans="1:2" ht="45" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A36" s="12" t="s">
         <v>120</v>
       </c>
-      <c r="B17" s="9" t="s">
-        <v>115</v>
-      </c>
-    </row>
-    <row r="18" spans="1:2" ht="45" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A18" s="12" t="s">
+      <c r="B36" s="11" t="s">
+        <v>119</v>
+      </c>
+    </row>
+    <row r="37" spans="1:2" ht="45" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A37" s="13" t="s">
         <v>121</v>
       </c>
-      <c r="B18" s="13" t="s">
+      <c r="B37" s="7" t="s">
         <v>122</v>
       </c>
     </row>
-    <row r="19" spans="1:2" ht="45" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A19" s="10" t="s">
+    <row r="38" spans="1:2" ht="45" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A38" s="12" t="s">
         <v>123</v>
       </c>
-      <c r="B19" s="9" t="s">
-        <v>104</v>
-      </c>
-    </row>
-    <row r="20" spans="1:2" ht="45" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A20" s="12" t="s">
-        <v>124</v>
-      </c>
-      <c r="B20" s="13" t="s">
+      <c r="B38" s="11" t="s">
+        <v>146</v>
+      </c>
+    </row>
+    <row r="39" spans="1:2" ht="45" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A39" s="13" t="s">
         <v>125</v>
       </c>
-    </row>
-    <row r="21" spans="1:2" ht="45" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A21" s="10" t="s">
-        <v>126</v>
-      </c>
-      <c r="B21" s="9" t="s">
+      <c r="B39" s="7" t="s">
+        <v>147</v>
+      </c>
+    </row>
+    <row r="40" spans="1:2" ht="45" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A40" s="12" t="s">
         <v>127</v>
       </c>
-    </row>
-    <row r="22" spans="1:2" ht="45" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A22" s="12" t="s">
+      <c r="B40" s="11" t="s">
+        <v>119</v>
+      </c>
+    </row>
+    <row r="41" spans="1:2" ht="45" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A41" s="13" t="s">
         <v>128</v>
       </c>
-      <c r="B22" s="13" t="s">
+      <c r="B41" s="7" t="s">
         <v>129</v>
       </c>
     </row>
-    <row r="23" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A23" s="19"/>
-      <c r="B23" s="19"/>
-    </row>
-    <row r="24" spans="1:2" ht="21" x14ac:dyDescent="0.25">
-      <c r="A24" s="15" t="s">
+    <row r="42" spans="1:2" ht="45" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A42" s="12" t="s">
         <v>130</v>
       </c>
-      <c r="B24" s="16"/>
-    </row>
-    <row r="25" spans="1:2" ht="18.75" x14ac:dyDescent="0.25">
-      <c r="A25" s="8" t="s">
-        <v>32</v>
-      </c>
-      <c r="B25" s="8" t="s">
-        <v>33</v>
-      </c>
-    </row>
-    <row r="26" spans="1:2" ht="45" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A26" s="10" t="s">
-        <v>96</v>
-      </c>
-      <c r="B26" s="9" t="s">
-        <v>115</v>
-      </c>
-    </row>
-    <row r="27" spans="1:2" ht="45" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A27" s="11" t="s">
-        <v>98</v>
-      </c>
-      <c r="B27" s="7" t="s">
+      <c r="B42" s="11" t="s">
+        <v>142</v>
+      </c>
+    </row>
+    <row r="43" spans="1:2" ht="45" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A43" s="13" t="s">
         <v>131</v>
       </c>
-    </row>
-    <row r="28" spans="1:2" ht="45" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A28" s="10" t="s">
-        <v>12</v>
-      </c>
-      <c r="B28" s="9" t="s">
-        <v>132</v>
-      </c>
-    </row>
-    <row r="29" spans="1:2" ht="45" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A29" s="11" t="s">
-        <v>39</v>
-      </c>
-      <c r="B29" s="7" t="s">
+      <c r="B43" s="7" t="s">
+        <v>148</v>
+      </c>
+    </row>
+    <row r="44" spans="1:2" ht="45" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A44" s="12" t="s">
         <v>133</v>
       </c>
-    </row>
-    <row r="30" spans="1:2" ht="45" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A30" s="10" t="s">
-        <v>25</v>
-      </c>
-      <c r="B30" s="9" t="s">
+      <c r="B44" s="11" t="s">
         <v>134</v>
       </c>
     </row>
-    <row r="31" spans="1:2" ht="45" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A31" s="11" t="s">
-        <v>103</v>
-      </c>
-      <c r="B31" s="7" t="s">
+    <row r="45" spans="1:2" ht="45" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A45" s="13" t="s">
         <v>135</v>
       </c>
-    </row>
-    <row r="32" spans="1:2" ht="45" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A32" s="10" t="s">
-        <v>105</v>
-      </c>
-      <c r="B32" s="9" t="s">
-        <v>136</v>
-      </c>
-    </row>
-    <row r="33" spans="1:2" ht="45" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A33" s="11" t="s">
-        <v>107</v>
-      </c>
-      <c r="B33" s="7" t="s">
-        <v>137</v>
-      </c>
-    </row>
-    <row r="34" spans="1:2" ht="45" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A34" s="10" t="s">
-        <v>109</v>
-      </c>
-      <c r="B34" s="9" t="s">
-        <v>138</v>
-      </c>
-    </row>
-    <row r="35" spans="1:2" ht="45" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A35" s="11" t="s">
-        <v>111</v>
-      </c>
-      <c r="B35" s="7" t="s">
-        <v>112</v>
-      </c>
-    </row>
-    <row r="36" spans="1:2" ht="45" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A36" s="10" t="s">
-        <v>113</v>
-      </c>
-      <c r="B36" s="9" t="s">
-        <v>112</v>
-      </c>
-    </row>
-    <row r="37" spans="1:2" ht="45" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A37" s="11" t="s">
-        <v>114</v>
-      </c>
-      <c r="B37" s="7" t="s">
-        <v>115</v>
-      </c>
-    </row>
-    <row r="38" spans="1:2" ht="45" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A38" s="10" t="s">
-        <v>116</v>
-      </c>
-      <c r="B38" s="9" t="s">
-        <v>139</v>
-      </c>
-    </row>
-    <row r="39" spans="1:2" ht="45" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A39" s="11" t="s">
-        <v>118</v>
-      </c>
-      <c r="B39" s="7" t="s">
-        <v>140</v>
-      </c>
-    </row>
-    <row r="40" spans="1:2" ht="45" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A40" s="10" t="s">
-        <v>120</v>
-      </c>
-      <c r="B40" s="9" t="s">
-        <v>112</v>
-      </c>
-    </row>
-    <row r="41" spans="1:2" ht="45" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A41" s="11" t="s">
-        <v>121</v>
-      </c>
-      <c r="B41" s="7" t="s">
-        <v>122</v>
-      </c>
-    </row>
-    <row r="42" spans="1:2" ht="45" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A42" s="10" t="s">
-        <v>123</v>
-      </c>
-      <c r="B42" s="9" t="s">
-        <v>135</v>
-      </c>
-    </row>
-    <row r="43" spans="1:2" ht="45" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A43" s="11" t="s">
-        <v>124</v>
-      </c>
-      <c r="B43" s="7" t="s">
-        <v>141</v>
-      </c>
-    </row>
-    <row r="44" spans="1:2" ht="45" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A44" s="10" t="s">
-        <v>126</v>
-      </c>
-      <c r="B44" s="9" t="s">
-        <v>127</v>
-      </c>
-    </row>
-    <row r="45" spans="1:2" ht="45" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A45" s="11" t="s">
-        <v>128</v>
-      </c>
       <c r="B45" s="7" t="s">
-        <v>142</v>
+        <v>149</v>
       </c>
     </row>
   </sheetData>

</xml_diff>